<commit_message>
Mark 10 shipped feature ideas as Done in the tracking sheet
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ClAuSy_Feature_Ideas.xlsx
+++ b/ClAuSy_Feature_Ideas.xlsx
@@ -628,8 +628,16 @@
           <t>Global search box to filter Directories list by label or path</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G6" s="3" t="inlineStr"/>
     </row>
     <row r="7" ht="30" customHeight="1">
@@ -651,8 +659,16 @@
           <t>Keyboard shortcuts (Ctrl+Z undo, Delete key, Ctrl+F search)</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr"/>
-      <c r="F7" s="4" t="inlineStr"/>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8" ht="30" customHeight="1">
@@ -697,8 +713,16 @@
           <t>Right-click context menu on rows (Open, Copy path, Remove)</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr"/>
-      <c r="F9" s="4" t="inlineStr"/>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10" ht="30" customHeight="1">
@@ -743,8 +767,16 @@
           <t>Remember window size/position between launches</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr"/>
-      <c r="F11" s="4" t="inlineStr"/>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G11" s="5" t="inlineStr"/>
     </row>
     <row r="12" ht="30" customHeight="1">
@@ -835,8 +867,16 @@
           <t>Collapsible legend / help panel to save vertical space</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr"/>
-      <c r="F15" s="4" t="inlineStr"/>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G15" s="5" t="inlineStr"/>
     </row>
     <row r="16" ht="30" customHeight="1">
@@ -927,8 +967,16 @@
           <t>Warn if a toggled-on directory doesn't exist on disk anymore</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr"/>
-      <c r="F19" s="4" t="inlineStr"/>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G19" s="5" t="inlineStr"/>
     </row>
     <row r="20" ht="30" customHeight="1">
@@ -950,8 +998,16 @@
           <t>Warn if the same directory is a parent of another tracked directory (overlap)</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr"/>
-      <c r="F20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G20" s="3" t="inlineStr"/>
     </row>
     <row r="21" ht="30" customHeight="1">
@@ -1686,8 +1742,16 @@
           <t>Word/line count + 'too long' warning for CLAUDE.md files (context budget)</t>
         </is>
       </c>
-      <c r="E52" s="2" t="inlineStr"/>
-      <c r="F52" s="2" t="inlineStr"/>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G52" s="3" t="inlineStr"/>
     </row>
     <row r="53" ht="30" customHeight="1">
@@ -1732,8 +1796,16 @@
           <t>Detect Hebrew/RTL content and confirm the required first line for Obsidian</t>
         </is>
       </c>
-      <c r="E54" s="2" t="inlineStr"/>
-      <c r="F54" s="2" t="inlineStr"/>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G54" s="3" t="inlineStr"/>
     </row>
     <row r="55" ht="30" customHeight="1">
@@ -2790,8 +2862,16 @@
           <t>'Report a confusing config' button that opens a pre-filled GitHub issue</t>
         </is>
       </c>
-      <c r="E100" s="2" t="inlineStr"/>
-      <c r="F100" s="2" t="inlineStr"/>
+      <c r="E100" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G100" s="3" t="inlineStr"/>
     </row>
     <row r="101" ht="30" customHeight="1">

</xml_diff>

<commit_message>
Add 30 research-grounded feature ideas (#101-130) to the roadmap sheet
Sourced from real anthropics/claude-code GitHub issues, a documented
YOLO-mode incident, and official docs — not speculation. Covers
permission-merge visibility, settings.json write-safety, the actual
CLAUDE.md line-count cliff (not word count), monorepo settings
discovery, and hook/subagent validation gaps.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ClAuSy_Feature_Ideas.xlsx
+++ b/ClAuSy_Feature_Ideas.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G101"/>
+  <dimension ref="A1:G131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2897,6 +2897,756 @@
       <c r="F101" s="4" t="inlineStr"/>
       <c r="G101" s="5" t="inlineStr"/>
     </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>101</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Warn prominently if permissions.defaultMode is bypassPermissions ('YOLO mode') — tied to a documented incident where it caused an rm -rf to wipe a user's home dir</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>102</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>One-click 'Deny secrets' preset — auto-add deny rules for .env, *.pem, *.key, id_rsa, credentials.json, etc.</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>103</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Safety / Trust</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Detect external changes to settings.json / claude_desktop_config.json since ClAuSy last read them, before writing (Claude Code itself has a known bug silently rewriting settings.json mid-session)</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>104</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Safety / Trust</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>On-write conflict detection: if a config file's on-disk content differs from what ClAuSy last loaded, show a diff and confirm before overwriting</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>105</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Effective merged-permissions viewer showing user/project/local scope merge for a directory, highlighting deny-wins-over-allow conflicts</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>106</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Warn when a deny rule and an allow rule both match the same path — deny always wins, but this isn't obvious to users</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>107</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Multi-source</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Detect .claude/settings.local.json and warn if it looks accidentally tracked in git instead of gitignored (it's meant to be personal/local-only)</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>108</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Multi-source</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Detect monorepo subfolders with their own .claude/settings.json that Claude Code won't discover automatically (no parent-directory traversal) and surface them</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>109</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>CLAUDE.md tools</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Rework the 'too long' warning to use line count (~100-200 lines) instead of word count — matches Claude's actual attention drop-off, not an arbitrary word cap</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>110</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>CLAUDE.md tools</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>'Context rot' checker — flag CLAUDE.md files that look auto-generated/bloated (repeated headers, huge bullet lists) as candidates for trimming</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>111</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Agents &amp; Routines</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Detect subagents with vague or overlapping description fields that could cause inconsistent auto-delegation</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>112</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Agents &amp; Routines</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>Flag subagent files that look stale/unused (best-effort, based on file mtime)</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>113</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Multi-source</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>Windows MSIX 'Edit Config' opens the wrong claude_desktop_config.json (documented bug) — show both possible paths and let the user confirm which one is actually active</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Reporting</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>'Config health check' report — one button that runs every warning (missing dirs, overlaps, RTL, too-long CLAUDE.md, bypassPermissions, deny/allow conflicts) at once</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Agents &amp; Routines</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>Validate hooks in settings.json against Claude Code's expected schema — hooks that look correctly configured can still silently fail to load</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>Warn when a hook runs a shell command that could be destructive (rm, git push --force, etc.)</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>Show which permission mode is currently effective (default/acceptEdits/plan/bypassPermissions) per tracked project, not just globally</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>'Safe defaults' one-click setup — allowlist read-only tools + deny secrets + no bypassPermissions, as a guided first-run preset</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Reporting</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>Session/weekly digest of permission changes since the last Execute</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>CLAUDE.md tools</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>Detect duplicate or conflicting instructions between global and project CLAUDE.md files, not just a raw diff</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>Detect and warn if Claude Code is being run with --dangerously-skip-permissions, if that's exposed anywhere ClAuSy can read</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Safety / Trust</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Backup rotation — keep the last N .bak files instead of overwriting a single one, for real rollback/audit capability</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>Visual scope inspector: show one directory's permission status merged across ALL settings.json layers (user, project, local) in a single row</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Onboarding / Docs</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>First-run 'safe defaults' wizard explaining permission fatigue and YOLO-mode risk, linking to Anthropic's own security guidance</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Multi-source</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Detect orphaned/duplicate MCP filesystem server entries across multiple claude_desktop_config.json install locations (Store vs. classic)</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Testing / Quality</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Regression test verifying apply_changes() never silently drops unrelated top-level keys (hooks, statusLine, enabledPlugins) — mirrors a real Claude Code bug</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Redact secret-looking directory names or content in any exported report</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>CLAUDE.md tools</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>Show an exact line-count badge (not just a boolean flag) so users can see how close a file is to the ~100-200 line danger zone</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Community</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>Link to Anthropic's official permission/security best-practices docs from the Explained tab</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>'Undo last Execute' — restore config files from the .bak snapshot with one click, not just in-app undo of unwritten toggles</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G101"/>
   <dataValidations count="2">

</xml_diff>

<commit_message>
Mark round 2's 10 shipped feature ideas as Done, update docs
Excel now has 130 total ideas (30 new, research-grounded ones added
this round) with 20 marked Done. CHANGELOG.md and the session log
reflect all 10 new security/safety features.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ClAuSy_Feature_Ideas.xlsx
+++ b/ClAuSy_Feature_Ideas.xlsx
@@ -2916,6 +2916,16 @@
           <t>Warn prominently if permissions.defaultMode is bypassPermissions ('YOLO mode') — tied to a documented incident where it caused an rm -rf to wipe a user's home dir</t>
         </is>
       </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G102" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
@@ -2941,6 +2951,16 @@
           <t>One-click 'Deny secrets' preset — auto-add deny rules for .env, *.pem, *.key, id_rsa, credentials.json, etc.</t>
         </is>
       </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G103" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
@@ -2966,6 +2986,16 @@
           <t>Detect external changes to settings.json / claude_desktop_config.json since ClAuSy last read them, before writing (Claude Code itself has a known bug silently rewriting settings.json mid-session)</t>
         </is>
       </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G104" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
@@ -3041,6 +3071,16 @@
           <t>Warn when a deny rule and an allow rule both match the same path — deny always wins, but this isn't obvious to users</t>
         </is>
       </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G107" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
@@ -3116,6 +3156,16 @@
           <t>Rework the 'too long' warning to use line count (~100-200 lines) instead of word count — matches Claude's actual attention drop-off, not an arbitrary word cap</t>
         </is>
       </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G110" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
@@ -3166,6 +3216,16 @@
           <t>Detect subagents with vague or overlapping description fields that could cause inconsistent auto-delegation</t>
         </is>
       </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G112" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
@@ -3216,6 +3276,16 @@
           <t>Windows MSIX 'Edit Config' opens the wrong claude_desktop_config.json (documented bug) — show both possible paths and let the user confirm which one is actually active</t>
         </is>
       </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G114" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
@@ -3366,6 +3436,16 @@
           <t>Session/weekly digest of permission changes since the last Execute</t>
         </is>
       </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G120" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
@@ -3441,6 +3521,16 @@
           <t>Backup rotation — keep the last N .bak files instead of overwriting a single one, for real rollback/audit capability</t>
         </is>
       </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G123" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
@@ -3639,6 +3729,16 @@
       <c r="D131" t="inlineStr">
         <is>
           <t>'Undo last Execute' — restore config files from the .bak snapshot with one click, not just in-app undo of unwritten toggles</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">

</xml_diff>

<commit_message>
Fix missing formatting on feature-ideas rows 101-130, add Date Added column
Round 2's append script skipped the fill/border/font/wrap/row-height styling
applied to rows 1-100, and left auto_filter stuck at A1:G101 (hiding rows
102-131 from the filter). Backfilled Date Added from git history: #1-100 and
#101-130 both landed 2026-09-14.
</commit_message>
<xml_diff>
--- a/ClAuSy_Feature_Ideas.xlsx
+++ b/ClAuSy_Feature_Ideas.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Ideas" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Feature Ideas'!$A$1:$G$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Feature Ideas'!$A$1:$H$131</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G131"/>
+  <dimension ref="A1:H131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -478,6 +478,7 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -516,6 +517,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Date Added</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="n">
@@ -539,6 +545,11 @@
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="3" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="4" t="n">
@@ -562,6 +573,11 @@
       <c r="E3" s="4" t="inlineStr"/>
       <c r="F3" s="4" t="inlineStr"/>
       <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="2" t="n">
@@ -585,6 +601,11 @@
       <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="3" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="4" t="n">
@@ -608,6 +629,11 @@
       <c r="E5" s="4" t="inlineStr"/>
       <c r="F5" s="4" t="inlineStr"/>
       <c r="G5" s="5" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="2" t="n">
@@ -639,6 +665,11 @@
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="4" t="n">
@@ -670,6 +701,11 @@
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="2" t="n">
@@ -693,6 +729,11 @@
       <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="3" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="4" t="n">
@@ -724,6 +765,11 @@
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="2" t="n">
@@ -747,6 +793,11 @@
       <c r="E10" s="2" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr"/>
       <c r="G10" s="3" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="4" t="n">
@@ -778,6 +829,11 @@
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr"/>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="2" t="n">
@@ -801,6 +857,11 @@
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="3" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="4" t="n">
@@ -824,6 +885,11 @@
       <c r="E13" s="4" t="inlineStr"/>
       <c r="F13" s="4" t="inlineStr"/>
       <c r="G13" s="5" t="inlineStr"/>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="2" t="n">
@@ -847,6 +913,11 @@
       <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
       <c r="G14" s="3" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="4" t="n">
@@ -878,6 +949,11 @@
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr"/>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="2" t="n">
@@ -901,6 +977,11 @@
       <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
       <c r="G16" s="3" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="4" t="n">
@@ -924,6 +1005,11 @@
       <c r="E17" s="4" t="inlineStr"/>
       <c r="F17" s="4" t="inlineStr"/>
       <c r="G17" s="5" t="inlineStr"/>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="2" t="n">
@@ -947,6 +1033,11 @@
       <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="3" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="4" t="n">
@@ -978,6 +1069,11 @@
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr"/>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="2" t="n">
@@ -1009,6 +1105,11 @@
         </is>
       </c>
       <c r="G20" s="3" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="4" t="n">
@@ -1032,6 +1133,11 @@
       <c r="E21" s="4" t="inlineStr"/>
       <c r="F21" s="4" t="inlineStr"/>
       <c r="G21" s="5" t="inlineStr"/>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="2" t="n">
@@ -1055,6 +1161,11 @@
       <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="3" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="4" t="n">
@@ -1078,6 +1189,11 @@
       <c r="E23" s="4" t="inlineStr"/>
       <c r="F23" s="4" t="inlineStr"/>
       <c r="G23" s="5" t="inlineStr"/>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="2" t="n">
@@ -1101,6 +1217,11 @@
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
       <c r="G24" s="3" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="4" t="n">
@@ -1124,6 +1245,11 @@
       <c r="E25" s="4" t="inlineStr"/>
       <c r="F25" s="4" t="inlineStr"/>
       <c r="G25" s="5" t="inlineStr"/>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="2" t="n">
@@ -1147,6 +1273,11 @@
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
       <c r="G26" s="3" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="4" t="n">
@@ -1170,6 +1301,11 @@
       <c r="E27" s="4" t="inlineStr"/>
       <c r="F27" s="4" t="inlineStr"/>
       <c r="G27" s="5" t="inlineStr"/>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="2" t="n">
@@ -1193,6 +1329,11 @@
       <c r="E28" s="2" t="inlineStr"/>
       <c r="F28" s="2" t="inlineStr"/>
       <c r="G28" s="3" t="inlineStr"/>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="4" t="n">
@@ -1216,6 +1357,11 @@
       <c r="E29" s="4" t="inlineStr"/>
       <c r="F29" s="4" t="inlineStr"/>
       <c r="G29" s="5" t="inlineStr"/>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="30" customHeight="1">
       <c r="A30" s="2" t="n">
@@ -1239,6 +1385,11 @@
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
       <c r="G30" s="3" t="inlineStr"/>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="4" t="n">
@@ -1262,6 +1413,11 @@
       <c r="E31" s="4" t="inlineStr"/>
       <c r="F31" s="4" t="inlineStr"/>
       <c r="G31" s="5" t="inlineStr"/>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="2" t="n">
@@ -1285,6 +1441,11 @@
       <c r="E32" s="2" t="inlineStr"/>
       <c r="F32" s="2" t="inlineStr"/>
       <c r="G32" s="3" t="inlineStr"/>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="4" t="n">
@@ -1308,6 +1469,11 @@
       <c r="E33" s="4" t="inlineStr"/>
       <c r="F33" s="4" t="inlineStr"/>
       <c r="G33" s="5" t="inlineStr"/>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="2" t="n">
@@ -1331,6 +1497,11 @@
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr"/>
       <c r="G34" s="3" t="inlineStr"/>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="4" t="n">
@@ -1354,6 +1525,11 @@
       <c r="E35" s="4" t="inlineStr"/>
       <c r="F35" s="4" t="inlineStr"/>
       <c r="G35" s="5" t="inlineStr"/>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="2" t="n">
@@ -1377,6 +1553,11 @@
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr"/>
       <c r="G36" s="3" t="inlineStr"/>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="30" customHeight="1">
       <c r="A37" s="4" t="n">
@@ -1400,6 +1581,11 @@
       <c r="E37" s="4" t="inlineStr"/>
       <c r="F37" s="4" t="inlineStr"/>
       <c r="G37" s="5" t="inlineStr"/>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="30" customHeight="1">
       <c r="A38" s="2" t="n">
@@ -1423,6 +1609,11 @@
       <c r="E38" s="2" t="inlineStr"/>
       <c r="F38" s="2" t="inlineStr"/>
       <c r="G38" s="3" t="inlineStr"/>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="30" customHeight="1">
       <c r="A39" s="4" t="n">
@@ -1446,6 +1637,11 @@
       <c r="E39" s="4" t="inlineStr"/>
       <c r="F39" s="4" t="inlineStr"/>
       <c r="G39" s="5" t="inlineStr"/>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="30" customHeight="1">
       <c r="A40" s="2" t="n">
@@ -1469,6 +1665,11 @@
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="2" t="inlineStr"/>
       <c r="G40" s="3" t="inlineStr"/>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="30" customHeight="1">
       <c r="A41" s="4" t="n">
@@ -1492,6 +1693,11 @@
       <c r="E41" s="4" t="inlineStr"/>
       <c r="F41" s="4" t="inlineStr"/>
       <c r="G41" s="5" t="inlineStr"/>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="30" customHeight="1">
       <c r="A42" s="2" t="n">
@@ -1515,6 +1721,11 @@
       <c r="E42" s="2" t="inlineStr"/>
       <c r="F42" s="2" t="inlineStr"/>
       <c r="G42" s="3" t="inlineStr"/>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="30" customHeight="1">
       <c r="A43" s="4" t="n">
@@ -1538,6 +1749,11 @@
       <c r="E43" s="4" t="inlineStr"/>
       <c r="F43" s="4" t="inlineStr"/>
       <c r="G43" s="5" t="inlineStr"/>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="30" customHeight="1">
       <c r="A44" s="2" t="n">
@@ -1561,6 +1777,11 @@
       <c r="E44" s="2" t="inlineStr"/>
       <c r="F44" s="2" t="inlineStr"/>
       <c r="G44" s="3" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="30" customHeight="1">
       <c r="A45" s="4" t="n">
@@ -1584,6 +1805,11 @@
       <c r="E45" s="4" t="inlineStr"/>
       <c r="F45" s="4" t="inlineStr"/>
       <c r="G45" s="5" t="inlineStr"/>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="30" customHeight="1">
       <c r="A46" s="2" t="n">
@@ -1607,6 +1833,11 @@
       <c r="E46" s="2" t="inlineStr"/>
       <c r="F46" s="2" t="inlineStr"/>
       <c r="G46" s="3" t="inlineStr"/>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="30" customHeight="1">
       <c r="A47" s="4" t="n">
@@ -1630,6 +1861,11 @@
       <c r="E47" s="4" t="inlineStr"/>
       <c r="F47" s="4" t="inlineStr"/>
       <c r="G47" s="5" t="inlineStr"/>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="30" customHeight="1">
       <c r="A48" s="2" t="n">
@@ -1653,6 +1889,11 @@
       <c r="E48" s="2" t="inlineStr"/>
       <c r="F48" s="2" t="inlineStr"/>
       <c r="G48" s="3" t="inlineStr"/>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="30" customHeight="1">
       <c r="A49" s="4" t="n">
@@ -1676,6 +1917,11 @@
       <c r="E49" s="4" t="inlineStr"/>
       <c r="F49" s="4" t="inlineStr"/>
       <c r="G49" s="5" t="inlineStr"/>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="2" t="n">
@@ -1699,6 +1945,11 @@
       <c r="E50" s="2" t="inlineStr"/>
       <c r="F50" s="2" t="inlineStr"/>
       <c r="G50" s="3" t="inlineStr"/>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="30" customHeight="1">
       <c r="A51" s="4" t="n">
@@ -1722,6 +1973,11 @@
       <c r="E51" s="4" t="inlineStr"/>
       <c r="F51" s="4" t="inlineStr"/>
       <c r="G51" s="5" t="inlineStr"/>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="30" customHeight="1">
       <c r="A52" s="2" t="n">
@@ -1753,6 +2009,11 @@
         </is>
       </c>
       <c r="G52" s="3" t="inlineStr"/>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="30" customHeight="1">
       <c r="A53" s="4" t="n">
@@ -1776,6 +2037,11 @@
       <c r="E53" s="4" t="inlineStr"/>
       <c r="F53" s="4" t="inlineStr"/>
       <c r="G53" s="5" t="inlineStr"/>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="30" customHeight="1">
       <c r="A54" s="2" t="n">
@@ -1807,6 +2073,11 @@
         </is>
       </c>
       <c r="G54" s="3" t="inlineStr"/>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="30" customHeight="1">
       <c r="A55" s="4" t="n">
@@ -1830,6 +2101,11 @@
       <c r="E55" s="4" t="inlineStr"/>
       <c r="F55" s="4" t="inlineStr"/>
       <c r="G55" s="5" t="inlineStr"/>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="30" customHeight="1">
       <c r="A56" s="2" t="n">
@@ -1853,6 +2129,11 @@
       <c r="E56" s="2" t="inlineStr"/>
       <c r="F56" s="2" t="inlineStr"/>
       <c r="G56" s="3" t="inlineStr"/>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="30" customHeight="1">
       <c r="A57" s="4" t="n">
@@ -1876,6 +2157,11 @@
       <c r="E57" s="4" t="inlineStr"/>
       <c r="F57" s="4" t="inlineStr"/>
       <c r="G57" s="5" t="inlineStr"/>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="30" customHeight="1">
       <c r="A58" s="2" t="n">
@@ -1899,6 +2185,11 @@
       <c r="E58" s="2" t="inlineStr"/>
       <c r="F58" s="2" t="inlineStr"/>
       <c r="G58" s="3" t="inlineStr"/>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="30" customHeight="1">
       <c r="A59" s="4" t="n">
@@ -1922,6 +2213,11 @@
       <c r="E59" s="4" t="inlineStr"/>
       <c r="F59" s="4" t="inlineStr"/>
       <c r="G59" s="5" t="inlineStr"/>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="30" customHeight="1">
       <c r="A60" s="2" t="n">
@@ -1945,6 +2241,11 @@
       <c r="E60" s="2" t="inlineStr"/>
       <c r="F60" s="2" t="inlineStr"/>
       <c r="G60" s="3" t="inlineStr"/>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="30" customHeight="1">
       <c r="A61" s="4" t="n">
@@ -1968,6 +2269,11 @@
       <c r="E61" s="4" t="inlineStr"/>
       <c r="F61" s="4" t="inlineStr"/>
       <c r="G61" s="5" t="inlineStr"/>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="30" customHeight="1">
       <c r="A62" s="2" t="n">
@@ -1991,6 +2297,11 @@
       <c r="E62" s="2" t="inlineStr"/>
       <c r="F62" s="2" t="inlineStr"/>
       <c r="G62" s="3" t="inlineStr"/>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="30" customHeight="1">
       <c r="A63" s="4" t="n">
@@ -2014,6 +2325,11 @@
       <c r="E63" s="4" t="inlineStr"/>
       <c r="F63" s="4" t="inlineStr"/>
       <c r="G63" s="5" t="inlineStr"/>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="30" customHeight="1">
       <c r="A64" s="2" t="n">
@@ -2037,6 +2353,11 @@
       <c r="E64" s="2" t="inlineStr"/>
       <c r="F64" s="2" t="inlineStr"/>
       <c r="G64" s="3" t="inlineStr"/>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="30" customHeight="1">
       <c r="A65" s="4" t="n">
@@ -2060,6 +2381,11 @@
       <c r="E65" s="4" t="inlineStr"/>
       <c r="F65" s="4" t="inlineStr"/>
       <c r="G65" s="5" t="inlineStr"/>
+      <c r="H65" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="30" customHeight="1">
       <c r="A66" s="2" t="n">
@@ -2083,6 +2409,11 @@
       <c r="E66" s="2" t="inlineStr"/>
       <c r="F66" s="2" t="inlineStr"/>
       <c r="G66" s="3" t="inlineStr"/>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="30" customHeight="1">
       <c r="A67" s="4" t="n">
@@ -2106,6 +2437,11 @@
       <c r="E67" s="4" t="inlineStr"/>
       <c r="F67" s="4" t="inlineStr"/>
       <c r="G67" s="5" t="inlineStr"/>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="30" customHeight="1">
       <c r="A68" s="2" t="n">
@@ -2129,6 +2465,11 @@
       <c r="E68" s="2" t="inlineStr"/>
       <c r="F68" s="2" t="inlineStr"/>
       <c r="G68" s="3" t="inlineStr"/>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="30" customHeight="1">
       <c r="A69" s="4" t="n">
@@ -2152,6 +2493,11 @@
       <c r="E69" s="4" t="inlineStr"/>
       <c r="F69" s="4" t="inlineStr"/>
       <c r="G69" s="5" t="inlineStr"/>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="30" customHeight="1">
       <c r="A70" s="2" t="n">
@@ -2175,6 +2521,11 @@
       <c r="E70" s="2" t="inlineStr"/>
       <c r="F70" s="2" t="inlineStr"/>
       <c r="G70" s="3" t="inlineStr"/>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="30" customHeight="1">
       <c r="A71" s="4" t="n">
@@ -2198,6 +2549,11 @@
       <c r="E71" s="4" t="inlineStr"/>
       <c r="F71" s="4" t="inlineStr"/>
       <c r="G71" s="5" t="inlineStr"/>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="30" customHeight="1">
       <c r="A72" s="2" t="n">
@@ -2221,6 +2577,11 @@
       <c r="E72" s="2" t="inlineStr"/>
       <c r="F72" s="2" t="inlineStr"/>
       <c r="G72" s="3" t="inlineStr"/>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="30" customHeight="1">
       <c r="A73" s="4" t="n">
@@ -2244,6 +2605,11 @@
       <c r="E73" s="4" t="inlineStr"/>
       <c r="F73" s="4" t="inlineStr"/>
       <c r="G73" s="5" t="inlineStr"/>
+      <c r="H73" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="30" customHeight="1">
       <c r="A74" s="2" t="n">
@@ -2267,6 +2633,11 @@
       <c r="E74" s="2" t="inlineStr"/>
       <c r="F74" s="2" t="inlineStr"/>
       <c r="G74" s="3" t="inlineStr"/>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="30" customHeight="1">
       <c r="A75" s="4" t="n">
@@ -2290,6 +2661,11 @@
       <c r="E75" s="4" t="inlineStr"/>
       <c r="F75" s="4" t="inlineStr"/>
       <c r="G75" s="5" t="inlineStr"/>
+      <c r="H75" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="30" customHeight="1">
       <c r="A76" s="2" t="n">
@@ -2313,6 +2689,11 @@
       <c r="E76" s="2" t="inlineStr"/>
       <c r="F76" s="2" t="inlineStr"/>
       <c r="G76" s="3" t="inlineStr"/>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="30" customHeight="1">
       <c r="A77" s="4" t="n">
@@ -2336,6 +2717,11 @@
       <c r="E77" s="4" t="inlineStr"/>
       <c r="F77" s="4" t="inlineStr"/>
       <c r="G77" s="5" t="inlineStr"/>
+      <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="30" customHeight="1">
       <c r="A78" s="2" t="n">
@@ -2359,6 +2745,11 @@
       <c r="E78" s="2" t="inlineStr"/>
       <c r="F78" s="2" t="inlineStr"/>
       <c r="G78" s="3" t="inlineStr"/>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="30" customHeight="1">
       <c r="A79" s="4" t="n">
@@ -2382,6 +2773,11 @@
       <c r="E79" s="4" t="inlineStr"/>
       <c r="F79" s="4" t="inlineStr"/>
       <c r="G79" s="5" t="inlineStr"/>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="30" customHeight="1">
       <c r="A80" s="2" t="n">
@@ -2405,6 +2801,11 @@
       <c r="E80" s="2" t="inlineStr"/>
       <c r="F80" s="2" t="inlineStr"/>
       <c r="G80" s="3" t="inlineStr"/>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="30" customHeight="1">
       <c r="A81" s="4" t="n">
@@ -2428,6 +2829,11 @@
       <c r="E81" s="4" t="inlineStr"/>
       <c r="F81" s="4" t="inlineStr"/>
       <c r="G81" s="5" t="inlineStr"/>
+      <c r="H81" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="30" customHeight="1">
       <c r="A82" s="2" t="n">
@@ -2451,6 +2857,11 @@
       <c r="E82" s="2" t="inlineStr"/>
       <c r="F82" s="2" t="inlineStr"/>
       <c r="G82" s="3" t="inlineStr"/>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="30" customHeight="1">
       <c r="A83" s="4" t="n">
@@ -2474,6 +2885,11 @@
       <c r="E83" s="4" t="inlineStr"/>
       <c r="F83" s="4" t="inlineStr"/>
       <c r="G83" s="5" t="inlineStr"/>
+      <c r="H83" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="30" customHeight="1">
       <c r="A84" s="2" t="n">
@@ -2497,6 +2913,11 @@
       <c r="E84" s="2" t="inlineStr"/>
       <c r="F84" s="2" t="inlineStr"/>
       <c r="G84" s="3" t="inlineStr"/>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="30" customHeight="1">
       <c r="A85" s="4" t="n">
@@ -2520,6 +2941,11 @@
       <c r="E85" s="4" t="inlineStr"/>
       <c r="F85" s="4" t="inlineStr"/>
       <c r="G85" s="5" t="inlineStr"/>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="30" customHeight="1">
       <c r="A86" s="2" t="n">
@@ -2543,6 +2969,11 @@
       <c r="E86" s="2" t="inlineStr"/>
       <c r="F86" s="2" t="inlineStr"/>
       <c r="G86" s="3" t="inlineStr"/>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="30" customHeight="1">
       <c r="A87" s="4" t="n">
@@ -2566,6 +2997,11 @@
       <c r="E87" s="4" t="inlineStr"/>
       <c r="F87" s="4" t="inlineStr"/>
       <c r="G87" s="5" t="inlineStr"/>
+      <c r="H87" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="30" customHeight="1">
       <c r="A88" s="2" t="n">
@@ -2589,6 +3025,11 @@
       <c r="E88" s="2" t="inlineStr"/>
       <c r="F88" s="2" t="inlineStr"/>
       <c r="G88" s="3" t="inlineStr"/>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="30" customHeight="1">
       <c r="A89" s="4" t="n">
@@ -2612,6 +3053,11 @@
       <c r="E89" s="4" t="inlineStr"/>
       <c r="F89" s="4" t="inlineStr"/>
       <c r="G89" s="5" t="inlineStr"/>
+      <c r="H89" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="30" customHeight="1">
       <c r="A90" s="2" t="n">
@@ -2635,6 +3081,11 @@
       <c r="E90" s="2" t="inlineStr"/>
       <c r="F90" s="2" t="inlineStr"/>
       <c r="G90" s="3" t="inlineStr"/>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="30" customHeight="1">
       <c r="A91" s="4" t="n">
@@ -2658,6 +3109,11 @@
       <c r="E91" s="4" t="inlineStr"/>
       <c r="F91" s="4" t="inlineStr"/>
       <c r="G91" s="5" t="inlineStr"/>
+      <c r="H91" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="30" customHeight="1">
       <c r="A92" s="2" t="n">
@@ -2681,6 +3137,11 @@
       <c r="E92" s="2" t="inlineStr"/>
       <c r="F92" s="2" t="inlineStr"/>
       <c r="G92" s="3" t="inlineStr"/>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="30" customHeight="1">
       <c r="A93" s="4" t="n">
@@ -2704,6 +3165,11 @@
       <c r="E93" s="4" t="inlineStr"/>
       <c r="F93" s="4" t="inlineStr"/>
       <c r="G93" s="5" t="inlineStr"/>
+      <c r="H93" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="30" customHeight="1">
       <c r="A94" s="2" t="n">
@@ -2727,6 +3193,11 @@
       <c r="E94" s="2" t="inlineStr"/>
       <c r="F94" s="2" t="inlineStr"/>
       <c r="G94" s="3" t="inlineStr"/>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="30" customHeight="1">
       <c r="A95" s="4" t="n">
@@ -2750,6 +3221,11 @@
       <c r="E95" s="4" t="inlineStr"/>
       <c r="F95" s="4" t="inlineStr"/>
       <c r="G95" s="5" t="inlineStr"/>
+      <c r="H95" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="30" customHeight="1">
       <c r="A96" s="2" t="n">
@@ -2773,6 +3249,11 @@
       <c r="E96" s="2" t="inlineStr"/>
       <c r="F96" s="2" t="inlineStr"/>
       <c r="G96" s="3" t="inlineStr"/>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="30" customHeight="1">
       <c r="A97" s="4" t="n">
@@ -2796,6 +3277,11 @@
       <c r="E97" s="4" t="inlineStr"/>
       <c r="F97" s="4" t="inlineStr"/>
       <c r="G97" s="5" t="inlineStr"/>
+      <c r="H97" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="30" customHeight="1">
       <c r="A98" s="2" t="n">
@@ -2819,6 +3305,11 @@
       <c r="E98" s="2" t="inlineStr"/>
       <c r="F98" s="2" t="inlineStr"/>
       <c r="G98" s="3" t="inlineStr"/>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="30" customHeight="1">
       <c r="A99" s="4" t="n">
@@ -2842,6 +3333,11 @@
       <c r="E99" s="4" t="inlineStr"/>
       <c r="F99" s="4" t="inlineStr"/>
       <c r="G99" s="5" t="inlineStr"/>
+      <c r="H99" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="30" customHeight="1">
       <c r="A100" s="2" t="n">
@@ -2873,6 +3369,11 @@
         </is>
       </c>
       <c r="G100" s="3" t="inlineStr"/>
+      <c r="H100" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="30" customHeight="1">
       <c r="A101" s="4" t="n">
@@ -2896,859 +3397,1054 @@
       <c r="E101" s="4" t="inlineStr"/>
       <c r="F101" s="4" t="inlineStr"/>
       <c r="G101" s="5" t="inlineStr"/>
-    </row>
-    <row r="102">
-      <c r="A102" t="n">
+      <c r="H101" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="30" customHeight="1">
+      <c r="A102" s="2" t="n">
         <v>101</v>
       </c>
-      <c r="B102" t="inlineStr">
+      <c r="B102" s="3" t="inlineStr">
         <is>
           <t>Security</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr">
+      <c r="C102" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D102" t="inlineStr">
+      <c r="D102" s="3" t="inlineStr">
         <is>
           <t>Warn prominently if permissions.defaultMode is bypassPermissions ('YOLO mode') — tied to a documented incident where it caused an rm -rf to wipe a user's home dir</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr">
+      <c r="E102" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F102" t="inlineStr">
+      <c r="F102" s="2" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G102" t="inlineStr">
+      <c r="G102" s="3" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="103">
-      <c r="A103" t="n">
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="30" customHeight="1">
+      <c r="A103" s="4" t="n">
         <v>102</v>
       </c>
-      <c r="B103" t="inlineStr">
+      <c r="B103" s="5" t="inlineStr">
         <is>
           <t>Security</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr">
+      <c r="C103" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D103" t="inlineStr">
+      <c r="D103" s="5" t="inlineStr">
         <is>
           <t>One-click 'Deny secrets' preset — auto-add deny rules for .env, *.pem, *.key, id_rsa, credentials.json, etc.</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr">
+      <c r="E103" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F103" t="inlineStr">
+      <c r="F103" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G103" t="inlineStr">
+      <c r="G103" s="5" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="104">
-      <c r="A104" t="n">
+      <c r="H103" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="30" customHeight="1">
+      <c r="A104" s="2" t="n">
         <v>103</v>
       </c>
-      <c r="B104" t="inlineStr">
+      <c r="B104" s="3" t="inlineStr">
         <is>
           <t>Safety / Trust</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr">
+      <c r="C104" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D104" t="inlineStr">
+      <c r="D104" s="3" t="inlineStr">
         <is>
           <t>Detect external changes to settings.json / claude_desktop_config.json since ClAuSy last read them, before writing (Claude Code itself has a known bug silently rewriting settings.json mid-session)</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr">
+      <c r="E104" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F104" t="inlineStr">
+      <c r="F104" s="2" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G104" t="inlineStr">
+      <c r="G104" s="3" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="105">
-      <c r="A105" t="n">
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="30" customHeight="1">
+      <c r="A105" s="4" t="n">
         <v>104</v>
       </c>
-      <c r="B105" t="inlineStr">
+      <c r="B105" s="5" t="inlineStr">
         <is>
           <t>Safety / Trust</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr">
+      <c r="C105" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D105" t="inlineStr">
+      <c r="D105" s="5" t="inlineStr">
         <is>
           <t>On-write conflict detection: if a config file's on-disk content differs from what ClAuSy last loaded, show a diff and confirm before overwriting</t>
         </is>
       </c>
-      <c r="G105" t="inlineStr">
+      <c r="E105" s="4" t="n"/>
+      <c r="F105" s="4" t="n"/>
+      <c r="G105" s="5" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="n">
+      <c r="H105" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="30" customHeight="1">
+      <c r="A106" s="2" t="n">
         <v>105</v>
       </c>
-      <c r="B106" t="inlineStr">
+      <c r="B106" s="3" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr">
+      <c r="C106" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D106" t="inlineStr">
+      <c r="D106" s="3" t="inlineStr">
         <is>
           <t>Effective merged-permissions viewer showing user/project/local scope merge for a directory, highlighting deny-wins-over-allow conflicts</t>
         </is>
       </c>
-      <c r="G106" t="inlineStr">
+      <c r="E106" s="2" t="n"/>
+      <c r="F106" s="2" t="n"/>
+      <c r="G106" s="3" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="107">
-      <c r="A107" t="n">
+      <c r="H106" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="30" customHeight="1">
+      <c r="A107" s="4" t="n">
         <v>106</v>
       </c>
-      <c r="B107" t="inlineStr">
+      <c r="B107" s="5" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr">
+      <c r="C107" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D107" s="5" t="inlineStr">
         <is>
           <t>Warn when a deny rule and an allow rule both match the same path — deny always wins, but this isn't obvious to users</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr">
+      <c r="E107" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F107" t="inlineStr">
+      <c r="F107" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G107" t="inlineStr">
+      <c r="G107" s="5" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="108">
-      <c r="A108" t="n">
+      <c r="H107" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="30" customHeight="1">
+      <c r="A108" s="2" t="n">
         <v>107</v>
       </c>
-      <c r="B108" t="inlineStr">
+      <c r="B108" s="3" t="inlineStr">
         <is>
           <t>Multi-source</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr">
+      <c r="C108" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr">
+      <c r="D108" s="3" t="inlineStr">
         <is>
           <t>Detect .claude/settings.local.json and warn if it looks accidentally tracked in git instead of gitignored (it's meant to be personal/local-only)</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr">
+      <c r="E108" s="2" t="n"/>
+      <c r="F108" s="2" t="n"/>
+      <c r="G108" s="3" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="109">
-      <c r="A109" t="n">
+      <c r="H108" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="30" customHeight="1">
+      <c r="A109" s="4" t="n">
         <v>108</v>
       </c>
-      <c r="B109" t="inlineStr">
+      <c r="B109" s="5" t="inlineStr">
         <is>
           <t>Multi-source</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr">
+      <c r="C109" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D109" s="5" t="inlineStr">
         <is>
           <t>Detect monorepo subfolders with their own .claude/settings.json that Claude Code won't discover automatically (no parent-directory traversal) and surface them</t>
         </is>
       </c>
-      <c r="G109" t="inlineStr">
+      <c r="E109" s="4" t="n"/>
+      <c r="F109" s="4" t="n"/>
+      <c r="G109" s="5" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="110">
-      <c r="A110" t="n">
+      <c r="H109" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="30" customHeight="1">
+      <c r="A110" s="2" t="n">
         <v>109</v>
       </c>
-      <c r="B110" t="inlineStr">
+      <c r="B110" s="3" t="inlineStr">
         <is>
           <t>CLAUDE.md tools</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr">
+      <c r="C110" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D110" t="inlineStr">
+      <c r="D110" s="3" t="inlineStr">
         <is>
           <t>Rework the 'too long' warning to use line count (~100-200 lines) instead of word count — matches Claude's actual attention drop-off, not an arbitrary word cap</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr">
+      <c r="E110" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr">
+      <c r="F110" s="2" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G110" t="inlineStr">
+      <c r="G110" s="3" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="111">
-      <c r="A111" t="n">
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="30" customHeight="1">
+      <c r="A111" s="4" t="n">
         <v>110</v>
       </c>
-      <c r="B111" t="inlineStr">
+      <c r="B111" s="5" t="inlineStr">
         <is>
           <t>CLAUDE.md tools</t>
         </is>
       </c>
-      <c r="C111" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D111" t="inlineStr">
+      <c r="C111" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D111" s="5" t="inlineStr">
         <is>
           <t>'Context rot' checker — flag CLAUDE.md files that look auto-generated/bloated (repeated headers, huge bullet lists) as candidates for trimming</t>
         </is>
       </c>
-      <c r="G111" t="inlineStr">
+      <c r="E111" s="4" t="n"/>
+      <c r="F111" s="4" t="n"/>
+      <c r="G111" s="5" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="112">
-      <c r="A112" t="n">
+      <c r="H111" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="30" customHeight="1">
+      <c r="A112" s="2" t="n">
         <v>111</v>
       </c>
-      <c r="B112" t="inlineStr">
+      <c r="B112" s="3" t="inlineStr">
         <is>
           <t>Agents &amp; Routines</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D112" t="inlineStr">
+      <c r="C112" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D112" s="3" t="inlineStr">
         <is>
           <t>Detect subagents with vague or overlapping description fields that could cause inconsistent auto-delegation</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr">
+      <c r="E112" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F112" t="inlineStr">
+      <c r="F112" s="2" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G112" t="inlineStr">
+      <c r="G112" s="3" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="113">
-      <c r="A113" t="n">
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="30" customHeight="1">
+      <c r="A113" s="4" t="n">
         <v>112</v>
       </c>
-      <c r="B113" t="inlineStr">
+      <c r="B113" s="5" t="inlineStr">
         <is>
           <t>Agents &amp; Routines</t>
         </is>
       </c>
-      <c r="C113" t="inlineStr">
+      <c r="C113" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="D113" t="inlineStr">
+      <c r="D113" s="5" t="inlineStr">
         <is>
           <t>Flag subagent files that look stale/unused (best-effort, based on file mtime)</t>
         </is>
       </c>
-      <c r="G113" t="inlineStr">
+      <c r="E113" s="4" t="n"/>
+      <c r="F113" s="4" t="n"/>
+      <c r="G113" s="5" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="114">
-      <c r="A114" t="n">
+      <c r="H113" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="30" customHeight="1">
+      <c r="A114" s="2" t="n">
         <v>113</v>
       </c>
-      <c r="B114" t="inlineStr">
+      <c r="B114" s="3" t="inlineStr">
         <is>
           <t>Multi-source</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr">
+      <c r="C114" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D114" t="inlineStr">
+      <c r="D114" s="3" t="inlineStr">
         <is>
           <t>Windows MSIX 'Edit Config' opens the wrong claude_desktop_config.json (documented bug) — show both possible paths and let the user confirm which one is actually active</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr">
+      <c r="E114" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F114" t="inlineStr">
+      <c r="F114" s="2" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G114" t="inlineStr">
+      <c r="G114" s="3" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="n">
+      <c r="H114" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="30" customHeight="1">
+      <c r="A115" s="4" t="n">
         <v>114</v>
       </c>
-      <c r="B115" t="inlineStr">
+      <c r="B115" s="5" t="inlineStr">
         <is>
           <t>Reporting</t>
         </is>
       </c>
-      <c r="C115" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D115" t="inlineStr">
+      <c r="C115" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D115" s="5" t="inlineStr">
         <is>
           <t>'Config health check' report — one button that runs every warning (missing dirs, overlaps, RTL, too-long CLAUDE.md, bypassPermissions, deny/allow conflicts) at once</t>
         </is>
       </c>
-      <c r="G115" t="inlineStr">
+      <c r="E115" s="4" t="n"/>
+      <c r="F115" s="4" t="n"/>
+      <c r="G115" s="5" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="116">
-      <c r="A116" t="n">
+      <c r="H115" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="30" customHeight="1">
+      <c r="A116" s="2" t="n">
         <v>115</v>
       </c>
-      <c r="B116" t="inlineStr">
+      <c r="B116" s="3" t="inlineStr">
         <is>
           <t>Agents &amp; Routines</t>
         </is>
       </c>
-      <c r="C116" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D116" t="inlineStr">
+      <c r="C116" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D116" s="3" t="inlineStr">
         <is>
           <t>Validate hooks in settings.json against Claude Code's expected schema — hooks that look correctly configured can still silently fail to load</t>
         </is>
       </c>
-      <c r="G116" t="inlineStr">
+      <c r="E116" s="2" t="n"/>
+      <c r="F116" s="2" t="n"/>
+      <c r="G116" s="3" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="117">
-      <c r="A117" t="n">
+      <c r="H116" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="30" customHeight="1">
+      <c r="A117" s="4" t="n">
         <v>116</v>
       </c>
-      <c r="B117" t="inlineStr">
+      <c r="B117" s="5" t="inlineStr">
         <is>
           <t>Security</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr">
+      <c r="C117" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D117" t="inlineStr">
+      <c r="D117" s="5" t="inlineStr">
         <is>
           <t>Warn when a hook runs a shell command that could be destructive (rm, git push --force, etc.)</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr">
+      <c r="E117" s="4" t="n"/>
+      <c r="F117" s="4" t="n"/>
+      <c r="G117" s="5" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="118">
-      <c r="A118" t="n">
+      <c r="H117" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="30" customHeight="1">
+      <c r="A118" s="2" t="n">
         <v>117</v>
       </c>
-      <c r="B118" t="inlineStr">
+      <c r="B118" s="3" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C118" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D118" t="inlineStr">
+      <c r="C118" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D118" s="3" t="inlineStr">
         <is>
           <t>Show which permission mode is currently effective (default/acceptEdits/plan/bypassPermissions) per tracked project, not just globally</t>
         </is>
       </c>
-      <c r="G118" t="inlineStr">
+      <c r="E118" s="2" t="n"/>
+      <c r="F118" s="2" t="n"/>
+      <c r="G118" s="3" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="119">
-      <c r="A119" t="n">
+      <c r="H118" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="30" customHeight="1">
+      <c r="A119" s="4" t="n">
         <v>118</v>
       </c>
-      <c r="B119" t="inlineStr">
+      <c r="B119" s="5" t="inlineStr">
         <is>
           <t>Security</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
+      <c r="C119" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D119" s="5" t="inlineStr">
         <is>
           <t>'Safe defaults' one-click setup — allowlist read-only tools + deny secrets + no bypassPermissions, as a guided first-run preset</t>
         </is>
       </c>
-      <c r="G119" t="inlineStr">
+      <c r="E119" s="4" t="n"/>
+      <c r="F119" s="4" t="n"/>
+      <c r="G119" s="5" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="120">
-      <c r="A120" t="n">
+      <c r="H119" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="30" customHeight="1">
+      <c r="A120" s="2" t="n">
         <v>119</v>
       </c>
-      <c r="B120" t="inlineStr">
+      <c r="B120" s="3" t="inlineStr">
         <is>
           <t>Reporting</t>
         </is>
       </c>
-      <c r="C120" t="inlineStr">
+      <c r="C120" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="D120" t="inlineStr">
+      <c r="D120" s="3" t="inlineStr">
         <is>
           <t>Session/weekly digest of permission changes since the last Execute</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr">
+      <c r="E120" s="2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F120" t="inlineStr">
+      <c r="F120" s="2" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G120" t="inlineStr">
+      <c r="G120" s="3" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="121">
-      <c r="A121" t="n">
+      <c r="H120" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="30" customHeight="1">
+      <c r="A121" s="4" t="n">
         <v>120</v>
       </c>
-      <c r="B121" t="inlineStr">
+      <c r="B121" s="5" t="inlineStr">
         <is>
           <t>CLAUDE.md tools</t>
         </is>
       </c>
-      <c r="C121" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D121" t="inlineStr">
+      <c r="C121" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D121" s="5" t="inlineStr">
         <is>
           <t>Detect duplicate or conflicting instructions between global and project CLAUDE.md files, not just a raw diff</t>
         </is>
       </c>
-      <c r="G121" t="inlineStr">
+      <c r="E121" s="4" t="n"/>
+      <c r="F121" s="4" t="n"/>
+      <c r="G121" s="5" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="122">
-      <c r="A122" t="n">
+      <c r="H121" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="30" customHeight="1">
+      <c r="A122" s="2" t="n">
         <v>121</v>
       </c>
-      <c r="B122" t="inlineStr">
+      <c r="B122" s="3" t="inlineStr">
         <is>
           <t>Security</t>
         </is>
       </c>
-      <c r="C122" t="inlineStr">
+      <c r="C122" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D122" t="inlineStr">
+      <c r="D122" s="3" t="inlineStr">
         <is>
           <t>Detect and warn if Claude Code is being run with --dangerously-skip-permissions, if that's exposed anywhere ClAuSy can read</t>
         </is>
       </c>
-      <c r="G122" t="inlineStr">
+      <c r="E122" s="2" t="n"/>
+      <c r="F122" s="2" t="n"/>
+      <c r="G122" s="3" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="123">
-      <c r="A123" t="n">
+      <c r="H122" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="30" customHeight="1">
+      <c r="A123" s="4" t="n">
         <v>122</v>
       </c>
-      <c r="B123" t="inlineStr">
+      <c r="B123" s="5" t="inlineStr">
         <is>
           <t>Safety / Trust</t>
         </is>
       </c>
-      <c r="C123" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D123" t="inlineStr">
+      <c r="C123" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D123" s="5" t="inlineStr">
         <is>
           <t>Backup rotation — keep the last N .bak files instead of overwriting a single one, for real rollback/audit capability</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr">
+      <c r="E123" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F123" t="inlineStr">
+      <c r="F123" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G123" t="inlineStr">
+      <c r="G123" s="5" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="124">
-      <c r="A124" t="n">
+      <c r="H123" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="30" customHeight="1">
+      <c r="A124" s="2" t="n">
         <v>123</v>
       </c>
-      <c r="B124" t="inlineStr">
+      <c r="B124" s="3" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C124" t="inlineStr">
+      <c r="C124" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D124" t="inlineStr">
+      <c r="D124" s="3" t="inlineStr">
         <is>
           <t>Visual scope inspector: show one directory's permission status merged across ALL settings.json layers (user, project, local) in a single row</t>
         </is>
       </c>
-      <c r="G124" t="inlineStr">
+      <c r="E124" s="2" t="n"/>
+      <c r="F124" s="2" t="n"/>
+      <c r="G124" s="3" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="125">
-      <c r="A125" t="n">
+      <c r="H124" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="30" customHeight="1">
+      <c r="A125" s="4" t="n">
         <v>124</v>
       </c>
-      <c r="B125" t="inlineStr">
+      <c r="B125" s="5" t="inlineStr">
         <is>
           <t>Onboarding / Docs</t>
         </is>
       </c>
-      <c r="C125" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D125" t="inlineStr">
+      <c r="C125" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D125" s="5" t="inlineStr">
         <is>
           <t>First-run 'safe defaults' wizard explaining permission fatigue and YOLO-mode risk, linking to Anthropic's own security guidance</t>
         </is>
       </c>
-      <c r="G125" t="inlineStr">
+      <c r="E125" s="4" t="n"/>
+      <c r="F125" s="4" t="n"/>
+      <c r="G125" s="5" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="126">
-      <c r="A126" t="n">
+      <c r="H125" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="30" customHeight="1">
+      <c r="A126" s="2" t="n">
         <v>125</v>
       </c>
-      <c r="B126" t="inlineStr">
+      <c r="B126" s="3" t="inlineStr">
         <is>
           <t>Multi-source</t>
         </is>
       </c>
-      <c r="C126" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D126" t="inlineStr">
+      <c r="C126" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D126" s="3" t="inlineStr">
         <is>
           <t>Detect orphaned/duplicate MCP filesystem server entries across multiple claude_desktop_config.json install locations (Store vs. classic)</t>
         </is>
       </c>
-      <c r="G126" t="inlineStr">
+      <c r="E126" s="2" t="n"/>
+      <c r="F126" s="2" t="n"/>
+      <c r="G126" s="3" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="127">
-      <c r="A127" t="n">
+      <c r="H126" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="30" customHeight="1">
+      <c r="A127" s="4" t="n">
         <v>126</v>
       </c>
-      <c r="B127" t="inlineStr">
+      <c r="B127" s="5" t="inlineStr">
         <is>
           <t>Testing / Quality</t>
         </is>
       </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D127" t="inlineStr">
+      <c r="C127" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D127" s="5" t="inlineStr">
         <is>
           <t>Regression test verifying apply_changes() never silently drops unrelated top-level keys (hooks, statusLine, enabledPlugins) — mirrors a real Claude Code bug</t>
         </is>
       </c>
-      <c r="G127" t="inlineStr">
+      <c r="E127" s="4" t="n"/>
+      <c r="F127" s="4" t="n"/>
+      <c r="G127" s="5" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="n">
+      <c r="H127" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="30" customHeight="1">
+      <c r="A128" s="2" t="n">
         <v>127</v>
       </c>
-      <c r="B128" t="inlineStr">
+      <c r="B128" s="3" t="inlineStr">
         <is>
           <t>Security</t>
         </is>
       </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr">
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D128" s="3" t="inlineStr">
         <is>
           <t>Redact secret-looking directory names or content in any exported report</t>
         </is>
       </c>
-      <c r="G128" t="inlineStr">
+      <c r="E128" s="2" t="n"/>
+      <c r="F128" s="2" t="n"/>
+      <c r="G128" s="3" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="n">
+      <c r="H128" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="30" customHeight="1">
+      <c r="A129" s="4" t="n">
         <v>128</v>
       </c>
-      <c r="B129" t="inlineStr">
+      <c r="B129" s="5" t="inlineStr">
         <is>
           <t>CLAUDE.md tools</t>
         </is>
       </c>
-      <c r="C129" t="inlineStr">
+      <c r="C129" s="4" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="D129" t="inlineStr">
+      <c r="D129" s="5" t="inlineStr">
         <is>
           <t>Show an exact line-count badge (not just a boolean flag) so users can see how close a file is to the ~100-200 line danger zone</t>
         </is>
       </c>
-      <c r="G129" t="inlineStr">
+      <c r="E129" s="4" t="n"/>
+      <c r="F129" s="4" t="n"/>
+      <c r="G129" s="5" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="n">
+      <c r="H129" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="30" customHeight="1">
+      <c r="A130" s="2" t="n">
         <v>129</v>
       </c>
-      <c r="B130" t="inlineStr">
+      <c r="B130" s="3" t="inlineStr">
         <is>
           <t>Community</t>
         </is>
       </c>
-      <c r="C130" t="inlineStr">
+      <c r="C130" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="D130" t="inlineStr">
+      <c r="D130" s="3" t="inlineStr">
         <is>
           <t>Link to Anthropic's official permission/security best-practices docs from the Explained tab</t>
         </is>
       </c>
-      <c r="G130" t="inlineStr">
+      <c r="E130" s="2" t="n"/>
+      <c r="F130" s="2" t="n"/>
+      <c r="G130" s="3" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="n">
+      <c r="H130" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="30" customHeight="1">
+      <c r="A131" s="4" t="n">
         <v>130</v>
       </c>
-      <c r="B131" t="inlineStr">
+      <c r="B131" s="5" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C131" t="inlineStr">
+      <c r="C131" s="4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="D131" t="inlineStr">
+      <c r="D131" s="5" t="inlineStr">
         <is>
           <t>'Undo last Execute' — restore config files from the .bak snapshot with one click, not just in-app undo of unwritten toggles</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr">
+      <c r="E131" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="F131" t="inlineStr">
+      <c r="F131" s="4" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="G131" t="inlineStr">
+      <c r="G131" s="5" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
         </is>
       </c>
+      <c r="H131" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G101"/>
+  <autoFilter ref="A1:H131"/>
   <dataValidations count="2">
     <dataValidation sqref="E2:E101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,Maybe"</formula1>

</xml_diff>

<commit_message>
Add 30 research-grounded feature ideas (#131-160) to the roadmap sheet
Sourced from real anthropics/claude-code GitHub issues (permission
precedence confusion, unsafe Bash wildcard matching, hook infinite-loop/log
explosions, orphaned MCP processes, force-push/branch-discipline incidents),
the ChainDrop npm worm (malicious hooks), and documented gaps in ClAuSy's
coverage (statusLine, output styles, plugin marketplaces).
</commit_message>
<xml_diff>
--- a/ClAuSy_Feature_Ideas.xlsx
+++ b/ClAuSy_Feature_Ideas.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Ideas" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Feature Ideas'!$A$1:$H$131</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Feature Ideas'!$A$1:$H$161</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H131"/>
+  <dimension ref="A1:H161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4443,8 +4443,968 @@
         </is>
       </c>
     </row>
+    <row r="132" ht="30" customHeight="1">
+      <c r="A132" s="2" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" s="3" t="inlineStr">
+        <is>
+          <t>Testing / Quality</t>
+        </is>
+      </c>
+      <c r="C132" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D132" s="3" t="inlineStr">
+        <is>
+          <t>Bundle a local settings.json schema and flag unrecognized/typo'd keys instead of silently accepting them.</t>
+        </is>
+      </c>
+      <c r="E132" s="2" t="n"/>
+      <c r="F132" s="2" t="n"/>
+      <c r="G132" s="3" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #94232, #82723 — no official schema; unknown keys accepted silently.</t>
+        </is>
+      </c>
+      <c r="H132" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="30" customHeight="1">
+      <c r="A133" s="4" t="n">
+        <v>132</v>
+      </c>
+      <c r="B133" s="5" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C133" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D133" s="5" t="inlineStr">
+        <is>
+          <t>Scan Bash allow rules for bare '*' / unsafe wildcards that could match shell operators (&amp;&amp;, ;, |) and flag as an injection risk.</t>
+        </is>
+      </c>
+      <c r="E133" s="4" t="n"/>
+      <c r="F133" s="4" t="n"/>
+      <c r="G133" s="5" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #40344.</t>
+        </is>
+      </c>
+      <c r="H133" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="30" customHeight="1">
+      <c r="A134" s="2" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" s="3" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="C134" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D134" s="3" t="inlineStr">
+        <is>
+          <t>Lint permission-rule wildcard syntax (catch 'npm *' vs correct 'npm:*') and auto-suggest the fix.</t>
+        </is>
+      </c>
+      <c r="E134" s="2" t="n"/>
+      <c r="F134" s="2" t="n"/>
+      <c r="G134" s="3" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #38223, #17619, #18961.</t>
+        </is>
+      </c>
+      <c r="H134" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="30" customHeight="1">
+      <c r="A135" s="4" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" s="5" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="C135" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D135" s="5" t="inlineStr">
+        <is>
+          <t>Watch settings.local.json for silent rewrites by Claude's own Edit tool that drop permission rules, and alert immediately.</t>
+        </is>
+      </c>
+      <c r="E135" s="4" t="n"/>
+      <c r="F135" s="4" t="n"/>
+      <c r="G135" s="5" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #41259.</t>
+        </is>
+      </c>
+      <c r="H135" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="30" customHeight="1">
+      <c r="A136" s="2" t="n">
+        <v>135</v>
+      </c>
+      <c r="B136" s="3" t="inlineStr">
+        <is>
+          <t>Multi-source</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D136" s="3" t="inlineStr">
+        <is>
+          <t>'Effective permissions' resolver view showing the merged allow/deny result across user/project/local/enterprise settings with which file actually wins.</t>
+        </is>
+      </c>
+      <c r="E136" s="2" t="n"/>
+      <c r="F136" s="2" t="n"/>
+      <c r="G136" s="3" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #18160, #19109, #21155 — repeated precedence-confusion reports.</t>
+        </is>
+      </c>
+      <c r="H136" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="30" customHeight="1">
+      <c r="A137" s="4" t="n">
+        <v>136</v>
+      </c>
+      <c r="B137" s="5" t="inlineStr">
+        <is>
+          <t>Multi-source</t>
+        </is>
+      </c>
+      <c r="C137" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D137" s="5" t="inlineStr">
+        <is>
+          <t>Detect and surface enterprise/managed-settings.json files that silently override user edits.</t>
+        </is>
+      </c>
+      <c r="E137" s="4" t="n"/>
+      <c r="F137" s="4" t="n"/>
+      <c r="G137" s="5" t="inlineStr">
+        <is>
+          <t>Same precedence-confusion issue class as the effective-permissions resolver idea.</t>
+        </is>
+      </c>
+      <c r="H137" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="30" customHeight="1">
+      <c r="A138" s="2" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="C138" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D138" s="3" t="inlineStr">
+        <is>
+          <t>Track bypassPermissions ('YOLO mode') on/off history per project with a persistent reminder banner showing how long it's been enabled.</t>
+        </is>
+      </c>
+      <c r="E138" s="2" t="n"/>
+      <c r="F138" s="2" t="n"/>
+      <c r="G138" s="3" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #93002 and documented YOLO-mode incidents (rm -rf on home/root).</t>
+        </is>
+      </c>
+      <c r="H138" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="30" customHeight="1">
+      <c r="A139" s="4" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" s="5" t="inlineStr">
+        <is>
+          <t>Multi-source</t>
+        </is>
+      </c>
+      <c r="C139" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D139" s="5" t="inlineStr">
+        <is>
+          <t>Flag known IDE-extension permission parity gaps (e.g. VSCode extension not honoring ~/.claude/settings.json).</t>
+        </is>
+      </c>
+      <c r="E139" s="4" t="n"/>
+      <c r="F139" s="4" t="n"/>
+      <c r="G139" s="5" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #29159.</t>
+        </is>
+      </c>
+      <c r="H139" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="30" customHeight="1">
+      <c r="A140" s="2" t="n">
+        <v>139</v>
+      </c>
+      <c r="B140" s="3" t="inlineStr">
+        <is>
+          <t>UX / Interface</t>
+        </is>
+      </c>
+      <c r="C140" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D140" s="3" t="inlineStr">
+        <is>
+          <t>Add a StatusLine manager tab — view, edit, and live-preview the statusLine command setting.</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="n"/>
+      <c r="F140" s="2" t="n"/>
+      <c r="G140" s="3" t="inlineStr">
+        <is>
+          <t>code.claude.com/docs/en/statusline — documented field ClAuSy doesn't cover.</t>
+        </is>
+      </c>
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="30" customHeight="1">
+      <c r="A141" s="4" t="n">
+        <v>140</v>
+      </c>
+      <c r="B141" s="5" t="inlineStr">
+        <is>
+          <t>UX / Interface</t>
+        </is>
+      </c>
+      <c r="C141" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D141" s="5" t="inlineStr">
+        <is>
+          <t>Add an Output Styles manager to list/switch/preview outputStyle.</t>
+        </is>
+      </c>
+      <c r="E141" s="4" t="n"/>
+      <c r="F141" s="4" t="n"/>
+      <c r="G141" s="5" t="inlineStr">
+        <is>
+          <t>Anthropic docs, output-styles feature — uncovered surface.</t>
+        </is>
+      </c>
+      <c r="H141" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="30" customHeight="1">
+      <c r="A142" s="2" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" s="3" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D142" s="3" t="inlineStr">
+        <is>
+          <t>Plugin &amp; marketplace inventory tab flagging marketplaces with auto-sync enabled (installs new plugins without consent).</t>
+        </is>
+      </c>
+      <c r="E142" s="2" t="n"/>
+      <c r="F142" s="2" t="n"/>
+      <c r="G142" s="3" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #37340; PromptArmor 'Hijacking Claude Code via Injected Marketplace Plugins.'</t>
+        </is>
+      </c>
+      <c r="H142" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="30" customHeight="1">
+      <c r="A143" s="4" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>Agents &amp; Hooks</t>
+        </is>
+      </c>
+      <c r="C143" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D143" s="5" t="inlineStr">
+        <is>
+          <t>Detect skill/plugin name collisions where an installed plugin shadows a custom subagent or skill.</t>
+        </is>
+      </c>
+      <c r="E143" s="4" t="n"/>
+      <c r="F143" s="4" t="n"/>
+      <c r="G143" s="5" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #40036.</t>
+        </is>
+      </c>
+      <c r="H143" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="30" customHeight="1">
+      <c r="A144" s="2" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C144" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D144" s="3" t="inlineStr">
+        <is>
+          <t>Scan hook shell commands for known-malicious patterns (pipe-to-shell, base64-decode-and-exec, obfuscated payloads).</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="n"/>
+      <c r="F144" s="2" t="n"/>
+      <c r="G144" s="3" t="inlineStr">
+        <is>
+          <t>ChainDrop npm worm, which planted a SessionStart hook to trigger on folder open.</t>
+        </is>
+      </c>
+      <c r="H144" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="30" customHeight="1">
+      <c r="A145" s="4" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" s="5" t="inlineStr">
+        <is>
+          <t>Agents &amp; Hooks</t>
+        </is>
+      </c>
+      <c r="C145" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D145" s="5" t="inlineStr">
+        <is>
+          <t>Detect hooks with no exit condition (Stop/UserPromptSubmit) that risk infinite retry loops or log explosions, and warn before saving.</t>
+        </is>
+      </c>
+      <c r="E145" s="4" t="n"/>
+      <c r="F145" s="4" t="n"/>
+      <c r="G145" s="5" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #10205, #17249, #55754, #58348.</t>
+        </is>
+      </c>
+      <c r="H145" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="30" customHeight="1">
+      <c r="A146" s="2" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>Agents &amp; Hooks</t>
+        </is>
+      </c>
+      <c r="C146" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="inlineStr">
+        <is>
+          <t>Find orphaned MCP server processes left running after Claude Code exits, and offer a one-click kill.</t>
+        </is>
+      </c>
+      <c r="E146" s="2" t="n"/>
+      <c r="F146" s="2" t="n"/>
+      <c r="G146" s="3" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #22612, #1935, #11778, #76306.</t>
+        </is>
+      </c>
+      <c r="H146" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="30" customHeight="1">
+      <c r="A147" s="4" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" s="5" t="inlineStr">
+        <is>
+          <t>Multi-source</t>
+        </is>
+      </c>
+      <c r="C147" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D147" s="5" t="inlineStr">
+        <is>
+          <t>MCP server reachability health-check (ping each configured server, flag dead/misconfigured ones, catch silently-dropped mcpServers blocks).</t>
+        </is>
+      </c>
+      <c r="E147" s="4" t="n"/>
+      <c r="F147" s="4" t="n"/>
+      <c r="G147" s="5" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #69084 — Desktop silently stripped the whole mcpServers block after an update.</t>
+        </is>
+      </c>
+      <c r="H147" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="30" customHeight="1">
+      <c r="A148" s="2" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>Git / Version Control</t>
+        </is>
+      </c>
+      <c r="C148" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D148" s="3" t="inlineStr">
+        <is>
+          <t>In Git Push tab, flag repos where the latest commit landed on main/master directly, against typical CLAUDE.md branch-discipline rules.</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="n"/>
+      <c r="F148" s="2" t="n"/>
+      <c r="G148" s="3" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #48474, #66109, #40695.</t>
+        </is>
+      </c>
+      <c r="H148" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="30" customHeight="1">
+      <c r="A149" s="4" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" s="5" t="inlineStr">
+        <is>
+          <t>Git / Version Control</t>
+        </is>
+      </c>
+      <c r="C149" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D149" s="5" t="inlineStr">
+        <is>
+          <t>Warn before push if local history was rewritten (amend/rebase) since the last known remote SHA.</t>
+        </is>
+      </c>
+      <c r="E149" s="4" t="n"/>
+      <c r="F149" s="4" t="n"/>
+      <c r="G149" s="5" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #16113, #32476.</t>
+        </is>
+      </c>
+      <c r="H149" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="30" customHeight="1">
+      <c r="A150" s="2" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" s="3" t="inlineStr">
+        <is>
+          <t>Git / Version Control</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D150" s="3" t="inlineStr">
+        <is>
+          <t>Flag unexpected/unintended new branch creation detected during a scan.</t>
+        </is>
+      </c>
+      <c r="E150" s="2" t="n"/>
+      <c r="F150" s="2" t="n"/>
+      <c r="G150" s="3" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #90600.</t>
+        </is>
+      </c>
+      <c r="H150" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="30" customHeight="1">
+      <c r="A151" s="4" t="n">
+        <v>150</v>
+      </c>
+      <c r="B151" s="5" t="inlineStr">
+        <is>
+          <t>Reporting</t>
+        </is>
+      </c>
+      <c r="C151" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D151" s="5" t="inlineStr">
+        <is>
+          <t>'Known-buggy-settings' radar — cross-reference the user's settings.json against a curated list of documented dead/no-op keys (e.g. teammateDefaultModel) and link the relevant issue.</t>
+        </is>
+      </c>
+      <c r="E151" s="4" t="n"/>
+      <c r="F151" s="4" t="n"/>
+      <c r="G151" s="5" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #82723.</t>
+        </is>
+      </c>
+      <c r="H151" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="30" customHeight="1">
+      <c r="A152" s="2" t="n">
+        <v>151</v>
+      </c>
+      <c r="B152" s="3" t="inlineStr">
+        <is>
+          <t>CLAUDE.md tools</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D152" s="3" t="inlineStr">
+        <is>
+          <t>Detect contradicting directives across global vs. project vs. subdirectory CLAUDE.md files (e.g. opposing formatting rules).</t>
+        </is>
+      </c>
+      <c r="E152" s="2" t="n"/>
+      <c r="F152" s="2" t="n"/>
+      <c r="G152" s="3" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #46724.</t>
+        </is>
+      </c>
+      <c r="H152" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="30" customHeight="1">
+      <c r="A153" s="4" t="n">
+        <v>152</v>
+      </c>
+      <c r="B153" s="5" t="inlineStr">
+        <is>
+          <t>CLAUDE.md tools</t>
+        </is>
+      </c>
+      <c r="C153" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D153" s="5" t="inlineStr">
+        <is>
+          <t>'Critical rule' pinning/reordering helper that surfaces a file's most important directives near the top, since instruction position affects adherence.</t>
+        </is>
+      </c>
+      <c r="E153" s="4" t="n"/>
+      <c r="F153" s="4" t="n"/>
+      <c r="G153" s="5" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #21119, #17530 — Claude ignores CLAUDE.md rules in roughly half of sessions.</t>
+        </is>
+      </c>
+      <c r="H153" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="30" customHeight="1">
+      <c r="A154" s="2" t="n">
+        <v>153</v>
+      </c>
+      <c r="B154" s="3" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D154" s="3" t="inlineStr">
+        <is>
+          <t>Cross-check permitted directories/paths against .gitignore to flag secret-pattern files that tools could still read despite being gitignored.</t>
+        </is>
+      </c>
+      <c r="E154" s="2" t="n"/>
+      <c r="F154" s="2" t="n"/>
+      <c r="G154" s="3" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #26286, #20609 — Glob/exploration ignoring .gitignore.</t>
+        </is>
+      </c>
+      <c r="H154" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="30" customHeight="1">
+      <c r="A155" s="4" t="n">
+        <v>154</v>
+      </c>
+      <c r="B155" s="5" t="inlineStr">
+        <is>
+          <t>Testing / Quality</t>
+        </is>
+      </c>
+      <c r="C155" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D155" s="5" t="inlineStr">
+        <is>
+          <t>Preflight disk-space check with a warning that low disk space silently prevents subagents/background tasks from running.</t>
+        </is>
+      </c>
+      <c r="E155" s="4" t="n"/>
+      <c r="F155" s="4" t="n"/>
+      <c r="G155" s="5" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #89603.</t>
+        </is>
+      </c>
+      <c r="H155" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="30" customHeight="1">
+      <c r="A156" s="2" t="n">
+        <v>155</v>
+      </c>
+      <c r="B156" s="3" t="inlineStr">
+        <is>
+          <t>Reporting</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D156" s="3" t="inlineStr">
+        <is>
+          <t>Installed Claude Code version/changelog watcher that surfaces settings.json-relevant changes on update.</t>
+        </is>
+      </c>
+      <c r="E156" s="2" t="n"/>
+      <c r="F156" s="2" t="n"/>
+      <c r="G156" s="3" t="inlineStr">
+        <is>
+          <t>General schema-drift issue class (#94232, #82723).</t>
+        </is>
+      </c>
+      <c r="H156" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="30" customHeight="1">
+      <c r="A157" s="4" t="n">
+        <v>156</v>
+      </c>
+      <c r="B157" s="5" t="inlineStr">
+        <is>
+          <t>Multi-source</t>
+        </is>
+      </c>
+      <c r="C157" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D157" s="5" t="inlineStr">
+        <is>
+          <t>Detect git worktrees of the same repo and group/dedupe their directory permission entries instead of treating each worktree as unrelated.</t>
+        </is>
+      </c>
+      <c r="E157" s="4" t="n"/>
+      <c r="F157" s="4" t="n"/>
+      <c r="G157" s="5" t="inlineStr">
+        <is>
+          <t>Real workflow friction — ClAuSy's own development already uses worktrees per session.</t>
+        </is>
+      </c>
+      <c r="H157" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" ht="30" customHeight="1">
+      <c r="A158" s="2" t="n">
+        <v>157</v>
+      </c>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D158" s="3" t="inlineStr">
+        <is>
+          <t>Deny-rule simulator — paste a sample command/path and show whether current allow/deny rules would actually block it.</t>
+        </is>
+      </c>
+      <c r="E158" s="2" t="n"/>
+      <c r="F158" s="2" t="n"/>
+      <c r="G158" s="3" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #27040 — deny rules silently not enforced.</t>
+        </is>
+      </c>
+      <c r="H158" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" ht="30" customHeight="1">
+      <c r="A159" s="4" t="n">
+        <v>158</v>
+      </c>
+      <c r="B159" s="5" t="inlineStr">
+        <is>
+          <t>Reporting</t>
+        </is>
+      </c>
+      <c r="C159" s="4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D159" s="5" t="inlineStr">
+        <is>
+          <t>Export a per-directory permission-mode matrix as CSV/PDF for audit/handoff purposes.</t>
+        </is>
+      </c>
+      <c r="E159" s="4" t="n"/>
+      <c r="F159" s="4" t="n"/>
+      <c r="G159" s="5" t="inlineStr">
+        <is>
+          <t>General enterprise/team audit need surfaced across permission-confusion issues.</t>
+        </is>
+      </c>
+      <c r="H159" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="30" customHeight="1">
+      <c r="A160" s="2" t="n">
+        <v>159</v>
+      </c>
+      <c r="B160" s="3" t="inlineStr">
+        <is>
+          <t>Testing / Quality</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D160" s="3" t="inlineStr">
+        <is>
+          <t>Regex/glob test harness — type a real Bash command and see exactly which permission rule matches it, resolving the documented prefix-vs-wildcard ambiguity.</t>
+        </is>
+      </c>
+      <c r="E160" s="2" t="n"/>
+      <c r="F160" s="2" t="n"/>
+      <c r="G160" s="3" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #18961, #17619 — doc contradictions on Bash permission matching.</t>
+        </is>
+      </c>
+      <c r="H160" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" ht="30" customHeight="1">
+      <c r="A161" s="4" t="n">
+        <v>160</v>
+      </c>
+      <c r="B161" s="5" t="inlineStr">
+        <is>
+          <t>Git / Version Control</t>
+        </is>
+      </c>
+      <c r="C161" s="4" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D161" s="5" t="inlineStr">
+        <is>
+          <t>Before a Push Selected/force-push action, show a preview of which commits would be discarded on the remote.</t>
+        </is>
+      </c>
+      <c r="E161" s="4" t="n"/>
+      <c r="F161" s="4" t="n"/>
+      <c r="G161" s="5" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #33402 — force-pushed over an existing private repo without asking.</t>
+        </is>
+      </c>
+      <c r="H161" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H131"/>
+  <autoFilter ref="A1:H161"/>
   <dataValidations count="2">
     <dataValidation sqref="E2:E101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,Maybe"</formula1>

</xml_diff>

<commit_message>
Mark round 3's 11 shipped feature ideas as Done in the tracking sheet
</commit_message>
<xml_diff>
--- a/ClAuSy_Feature_Ideas.xlsx
+++ b/ClAuSy_Feature_Ideas.xlsx
@@ -2798,8 +2798,16 @@
           <t>Detect and warn if a granted directory is a sensitive system path (System32, /etc, ~/.ssh)</t>
         </is>
       </c>
-      <c r="E80" s="2" t="inlineStr"/>
-      <c r="F80" s="2" t="inlineStr"/>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G80" s="3" t="inlineStr"/>
       <c r="H80" s="2" t="inlineStr">
         <is>
@@ -4462,8 +4470,16 @@
           <t>Bundle a local settings.json schema and flag unrecognized/typo'd keys instead of silently accepting them.</t>
         </is>
       </c>
-      <c r="E132" s="2" t="n"/>
-      <c r="F132" s="2" t="n"/>
+      <c r="E132" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F132" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G132" s="3" t="inlineStr">
         <is>
           <t>GitHub anthropics/claude-code #94232, #82723 — no official schema; unknown keys accepted silently.</t>
@@ -4654,8 +4670,16 @@
           <t>Track bypassPermissions ('YOLO mode') on/off history per project with a persistent reminder banner showing how long it's been enabled.</t>
         </is>
       </c>
-      <c r="E138" s="2" t="n"/>
-      <c r="F138" s="2" t="n"/>
+      <c r="E138" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F138" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G138" s="3" t="inlineStr">
         <is>
           <t>GitHub anthropics/claude-code #93002 and documented YOLO-mode incidents (rm -rf on home/root).</t>
@@ -4846,8 +4870,16 @@
           <t>Scan hook shell commands for known-malicious patterns (pipe-to-shell, base64-decode-and-exec, obfuscated payloads).</t>
         </is>
       </c>
-      <c r="E144" s="2" t="n"/>
-      <c r="F144" s="2" t="n"/>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G144" s="3" t="inlineStr">
         <is>
           <t>ChainDrop npm worm, which planted a SessionStart hook to trigger on folder open.</t>
@@ -4878,8 +4910,16 @@
           <t>Detect hooks with no exit condition (Stop/UserPromptSubmit) that risk infinite retry loops or log explosions, and warn before saving.</t>
         </is>
       </c>
-      <c r="E145" s="4" t="n"/>
-      <c r="F145" s="4" t="n"/>
+      <c r="E145" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F145" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G145" s="5" t="inlineStr">
         <is>
           <t>GitHub anthropics/claude-code #10205, #17249, #55754, #58348.</t>
@@ -4974,8 +5014,16 @@
           <t>In Git Push tab, flag repos where the latest commit landed on main/master directly, against typical CLAUDE.md branch-discipline rules.</t>
         </is>
       </c>
-      <c r="E148" s="2" t="n"/>
-      <c r="F148" s="2" t="n"/>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G148" s="3" t="inlineStr">
         <is>
           <t>GitHub anthropics/claude-code #48474, #66109, #40695.</t>
@@ -5038,8 +5086,16 @@
           <t>Flag unexpected/unintended new branch creation detected during a scan.</t>
         </is>
       </c>
-      <c r="E150" s="2" t="n"/>
-      <c r="F150" s="2" t="n"/>
+      <c r="E150" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G150" s="3" t="inlineStr">
         <is>
           <t>GitHub anthropics/claude-code #90600.</t>
@@ -5166,8 +5222,16 @@
           <t>Cross-check permitted directories/paths against .gitignore to flag secret-pattern files that tools could still read despite being gitignored.</t>
         </is>
       </c>
-      <c r="E154" s="2" t="n"/>
-      <c r="F154" s="2" t="n"/>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F154" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G154" s="3" t="inlineStr">
         <is>
           <t>GitHub anthropics/claude-code #26286, #20609 — Glob/exploration ignoring .gitignore.</t>
@@ -5294,8 +5358,16 @@
           <t>Deny-rule simulator — paste a sample command/path and show whether current allow/deny rules would actually block it.</t>
         </is>
       </c>
-      <c r="E158" s="2" t="n"/>
-      <c r="F158" s="2" t="n"/>
+      <c r="E158" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F158" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G158" s="3" t="inlineStr">
         <is>
           <t>GitHub anthropics/claude-code #27040 — deny rules silently not enforced.</t>
@@ -5358,8 +5430,16 @@
           <t>Regex/glob test harness — type a real Bash command and see exactly which permission rule matches it, resolving the documented prefix-vs-wildcard ambiguity.</t>
         </is>
       </c>
-      <c r="E160" s="2" t="n"/>
-      <c r="F160" s="2" t="n"/>
+      <c r="E160" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F160" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G160" s="3" t="inlineStr">
         <is>
           <t>GitHub anthropics/claude-code #18961, #17619 — doc contradictions on Bash permission matching.</t>
@@ -5390,8 +5470,16 @@
           <t>Before a Push Selected/force-push action, show a preview of which commits would be discarded on the remote.</t>
         </is>
       </c>
-      <c r="E161" s="4" t="n"/>
-      <c r="F161" s="4" t="n"/>
+      <c r="E161" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F161" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G161" s="5" t="inlineStr">
         <is>
           <t>GitHub anthropics/claude-code #33402 — force-pushed over an existing private repo without asking.</t>

</xml_diff>

<commit_message>
Mark 3 already-shipped ideas as Done in the tracking sheet
#17 (Restore-from-.bak button), #30 (visual permission-conflict detector),
and #104 (on-write conflict detection with a confirm dialog) were all
implemented in earlier rounds but never marked Done, risking duplicate
re-implementation.
</commit_message>
<xml_diff>
--- a/ClAuSy_Feature_Ideas.xlsx
+++ b/ClAuSy_Feature_Ideas.xlsx
@@ -1030,9 +1030,21 @@
           <t>Restore-from-.bak button in Settings if a write goes wrong</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr"/>
-      <c r="F18" s="2" t="inlineStr"/>
-      <c r="G18" s="3" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> [Confirmed already shipped in an earlier round — tracking sheet was out of date.]</t>
+        </is>
+      </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
           <t>2026-09-14</t>
@@ -1410,9 +1422,21 @@
           <t>Visual permission-conflict detector (e.g. allow + deny on the same path)</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr"/>
-      <c r="F31" s="4" t="inlineStr"/>
-      <c r="G31" s="5" t="inlineStr"/>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> [Confirmed already shipped in an earlier round — tracking sheet was out of date.]</t>
+        </is>
+      </c>
       <c r="H31" s="4" t="inlineStr">
         <is>
           <t>2026-09-14</t>
@@ -3550,11 +3574,19 @@
           <t>On-write conflict detection: if a config file's on-disk content differs from what ClAuSy last loaded, show a diff and confirm before overwriting</t>
         </is>
       </c>
-      <c r="E105" s="4" t="n"/>
-      <c r="F105" s="4" t="n"/>
+      <c r="E105" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F105" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G105" s="5" t="inlineStr">
         <is>
-          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
+          <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md. [Confirmed already shipped in an earlier round — tracking sheet was out of date.]</t>
         </is>
       </c>
       <c r="H105" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Mark round 4's 8 shipped feature ideas as Done in the tracking sheet
</commit_message>
<xml_diff>
--- a/ClAuSy_Feature_Ideas.xlsx
+++ b/ClAuSy_Feature_Ideas.xlsx
@@ -3614,8 +3614,16 @@
           <t>Effective merged-permissions viewer showing user/project/local scope merge for a directory, highlighting deny-wins-over-allow conflicts</t>
         </is>
       </c>
-      <c r="E106" s="2" t="n"/>
-      <c r="F106" s="2" t="n"/>
+      <c r="E106" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F106" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G106" s="3" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
@@ -3686,8 +3694,16 @@
           <t>Detect .claude/settings.local.json and warn if it looks accidentally tracked in git instead of gitignored (it's meant to be personal/local-only)</t>
         </is>
       </c>
-      <c r="E108" s="2" t="n"/>
-      <c r="F108" s="2" t="n"/>
+      <c r="E108" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F108" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G108" s="3" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
@@ -3998,8 +4014,16 @@
           <t>Warn when a hook runs a shell command that could be destructive (rm, git push --force, etc.)</t>
         </is>
       </c>
-      <c r="E117" s="4" t="n"/>
-      <c r="F117" s="4" t="n"/>
+      <c r="E117" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F117" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G117" s="5" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
@@ -4238,8 +4262,16 @@
           <t>Visual scope inspector: show one directory's permission status merged across ALL settings.json layers (user, project, local) in a single row</t>
         </is>
       </c>
-      <c r="E124" s="2" t="n"/>
-      <c r="F124" s="2" t="n"/>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G124" s="3" t="inlineStr">
         <is>
           <t>Grounded in real anthropics/claude-code GitHub issues, documented incidents, and official docs — see research notes in CHANGELOG/CLAUDE.md.</t>
@@ -4542,8 +4574,16 @@
           <t>Scan Bash allow rules for bare '*' / unsafe wildcards that could match shell operators (&amp;&amp;, ;, |) and flag as an injection risk.</t>
         </is>
       </c>
-      <c r="E133" s="4" t="n"/>
-      <c r="F133" s="4" t="n"/>
+      <c r="E133" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F133" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G133" s="5" t="inlineStr">
         <is>
           <t>GitHub anthropics/claude-code #40344.</t>
@@ -4606,8 +4646,16 @@
           <t>Watch settings.local.json for silent rewrites by Claude's own Edit tool that drop permission rules, and alert immediately.</t>
         </is>
       </c>
-      <c r="E135" s="4" t="n"/>
-      <c r="F135" s="4" t="n"/>
+      <c r="E135" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F135" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G135" s="5" t="inlineStr">
         <is>
           <t>GitHub anthropics/claude-code #41259.</t>
@@ -4638,8 +4686,16 @@
           <t>'Effective permissions' resolver view showing the merged allow/deny result across user/project/local/enterprise settings with which file actually wins.</t>
         </is>
       </c>
-      <c r="E136" s="2" t="n"/>
-      <c r="F136" s="2" t="n"/>
+      <c r="E136" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F136" s="2" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G136" s="3" t="inlineStr">
         <is>
           <t>GitHub anthropics/claude-code #18160, #19109, #21155 — repeated precedence-confusion reports.</t>
@@ -5086,8 +5142,16 @@
           <t>Warn before push if local history was rewritten (amend/rebase) since the last known remote SHA.</t>
         </is>
       </c>
-      <c r="E149" s="4" t="n"/>
-      <c r="F149" s="4" t="n"/>
+      <c r="E149" s="4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F149" s="4" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G149" s="5" t="inlineStr">
         <is>
           <t>GitHub anthropics/claude-code #16113, #32476.</t>

</xml_diff>

<commit_message>
Add user's launch-readiness note as roadmap item #161
Preserves a note added directly to the tracking sheet during round 4 (a git
pull would otherwise have overwritten it): making the product fully
production-ready end-to-end, and keeping the repo private for now.
</commit_message>
<xml_diff>
--- a/ClAuSy_Feature_Ideas.xlsx
+++ b/ClAuSy_Feature_Ideas.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Ideas" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Feature Ideas'!$A$1:$H$161</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Feature Ideas'!$A$1:$H$162</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H161"/>
+  <dimension ref="A1:H162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5587,8 +5587,40 @@
         </is>
       </c>
     </row>
+    <row r="162" ht="30" customHeight="1">
+      <c r="A162" s="2" t="n">
+        <v>161</v>
+      </c>
+      <c r="B162" s="3" t="inlineStr">
+        <is>
+          <t>Meta / Launch Readiness</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D162" s="3" t="inlineStr">
+        <is>
+          <t>הכי חשוב מכולם - להפוך את המוצר מא' עד ת' שיהייה מוכן לצאת כמוצר. וגם שיהייה בריפו פרטי בינתיים</t>
+        </is>
+      </c>
+      <c r="E162" s="2" t="n"/>
+      <c r="F162" s="2" t="n"/>
+      <c r="G162" s="3" t="inlineStr">
+        <is>
+          <t>Added directly by the user in the tracking sheet — production readiness and repo-visibility decision.</t>
+        </is>
+      </c>
+      <c r="H162" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H161"/>
+  <autoFilter ref="A1:H162"/>
   <dataValidations count="2">
     <dataValidation sqref="E2:E101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,Maybe"</formula1>

</xml_diff>

<commit_message>
Remove roadmap #161 (private-repo note) — decided to stay public and free
</commit_message>
<xml_diff>
--- a/ClAuSy_Feature_Ideas.xlsx
+++ b/ClAuSy_Feature_Ideas.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Ideas" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Feature Ideas'!$A$1:$H$162</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Feature Ideas'!$A$1:$H$161</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H162"/>
+  <dimension ref="A1:H161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5587,40 +5587,9 @@
         </is>
       </c>
     </row>
-    <row r="162" ht="30" customHeight="1">
-      <c r="A162" s="2" t="n">
-        <v>161</v>
-      </c>
-      <c r="B162" s="3" t="inlineStr">
-        <is>
-          <t>Meta / Launch Readiness</t>
-        </is>
-      </c>
-      <c r="C162" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D162" s="3" t="inlineStr">
-        <is>
-          <t>הכי חשוב מכולם - להפוך את המוצר מא' עד ת' שיהייה מוכן לצאת כמוצר. וגם שיהייה בריפו פרטי בינתיים</t>
-        </is>
-      </c>
-      <c r="E162" s="2" t="n"/>
-      <c r="F162" s="2" t="n"/>
-      <c r="G162" s="3" t="inlineStr">
-        <is>
-          <t>Added directly by the user in the tracking sheet — production readiness and repo-visibility decision.</t>
-        </is>
-      </c>
-      <c r="H162" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-16</t>
-        </is>
-      </c>
-    </row>
+    <row r="162" ht="30" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A1:H162"/>
+  <autoFilter ref="A1:H161"/>
   <dataValidations count="2">
     <dataValidation sqref="E2:E101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,Maybe"</formula1>

</xml_diff>

<commit_message>
Add 30 round-5 feature ideas (#161-190) from MCP/skills/security research
</commit_message>
<xml_diff>
--- a/ClAuSy_Feature_Ideas.xlsx
+++ b/ClAuSy_Feature_Ideas.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H161"/>
+  <dimension ref="A1:H191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5587,7 +5587,906 @@
         </is>
       </c>
     </row>
-    <row r="162" ht="30" customHeight="1"/>
+    <row r="162" ht="30" customHeight="1">
+      <c r="A162" t="n">
+        <v>161</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Precedence blind-spot detector: warn when defaultMode: bypassPermissions is set but a higher-precedence settings file also defines a permissions block, silently overriding it.</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #55507, #34923 — defaultMode silently dropped by permissions-block precedence merge bug</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>162</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>Stale-permission-cache warning: flag that editing settings.local.json directly while Claude Code is running may not take effect until restart.</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #41259 — Edit-tool modifications to settings.local.json stop being respected mid-session</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>163</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>New MCP Servers tab: list servers configured across .mcp.json (project), ~/.claude.json (user, mcpServers key), and .claude/settings.json, since the latter doesn't actually work for MCP.</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #37165, #4976, #42860 — .claude.json undocumented/unknown as an MCP config location</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>164</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>MCP server config validator — check server command exists on PATH and required env vars are set, before the user restarts Claude Code.</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #29824 — no way to validate config before restarting, silent failures</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>165</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>MCP</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>MCP precedence explainer — for a server name defined in multiple scopes (user/project/local), show which one wins, like the existing permission simulator.</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #29824, #15797 — multiple valid MCP config locations with no visibility into what's loaded</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>166</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Plugins / Skills</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>New Skills tab: list skills found in .claude/skills/ and ~/.claude/skills/, cross-checked against CLAUDE_CONFIG_DIR if set.</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #31649 — skills lookup hardcoded to ~/.claude/skills, ignores CLAUDE_CONFIG_DIR</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="n">
+        <v>167</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Plugins / Skills</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>Flag skills granted only via additionalDirectories in settings vs. --add-dir, since only the latter reliably loads skills.</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #37553 — skills not loaded from additionalDirectories, but loaded via --add-dir</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>168</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Plugins / Skills</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Managed-skills-path health check — verify any referenced managed skills directory actually exists; a missing one aborts all user-skill loading.</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #20576 — ENOENT on managed skills dir aborts entire skill-loading process</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>169</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Marketplace plugin hook auditor — extend find_dangerous_hook_commands() to also scan installed plugin manifests under ~/.claude/plugins/ for injected hook definitions.</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>PromptArmor — Hijacking Claude Code via Injected Marketplace Plugins; malicious plugins add hooks silently</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>170</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>Plugin marketplace registry viewer — list configured marketplace sources and flag any that aren't the official Anthropic marketplace for manual review.</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>Same PromptArmor disclosure — unofficial/injected marketplace sources as an attack vector</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>171</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>Supply-chain hook-diff alert — when a tracked repo's .claude/settings.json hooks section changes between the last-seen commit and HEAD (e.g. after a git pull), surface a dedicated high-visibility warning distinct from the generic external-change dialog.</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>Check Point CVE-2025-59536 — malicious repo hooks in settings.json execute at session init before any trust prompt</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>172</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>Repo-hooks-changed-by-someone-else badge in Git Push tab — flag if HEAD's hooks differ from the hooks at the last commit authored by the current git user (heuristic for hooks added in a commit you didn't write).</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>Same CVE-2025-59536 class of attack — same-repo hook injection via PR/contributor</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>173</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>Zero-deny + bypass-mode combo alert — separate from the existing YOLO-duration banner, specifically flag the combination of bypassPermissions with an empty deny list as unusually risky.</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>Derived from #27040/#34923 deny-enforcement bug pattern + general bypass-mode risk reports</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>174</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>CLAUDE.md / Docs</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>Context-budget dashboard on the CLAUDE.md Map tab — sum estimated tokens across the full chain (enterprise + user + project + parent CLAUDE.md + .claude/rules/*.md) that get reloaded every turn.</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #46526, #52979 — CLAUDE.md/rules/MCP schemas retransmitted every turn, large fixed token overhead</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>175</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>CLAUDE.md / Docs</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>Index .claude/rules/*.md files alongside CLAUDE.md in the Map tab — currently untracked, but they're a distinct doc source with the same subagent-blind-spot problem.</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #29423 — Task subagents don't load project CLAUDE.md or .claude/rules/*.md</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>176</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>CLAUDE.md / Docs</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>Enterprise/managed-settings.json awareness — detect and display the system-level managed-settings file (top precedence, can silently override user choices) if present.</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #86046 — Managed.settings.json interaction bugs</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>177</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Agents / Hooks</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Subagent CLAUDE.md-blind-spot banner in Agents &amp; Routines tab — flag subagent definitions likely relying on project conventions the subagent won't see (no CLAUDE.md read instruction in description, project has a non-trivial CLAUDE.md).</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #34572, #29423 — subagents don't inherit CLAUDE.md/rules, silently apply their own interpretation</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>178</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Agents / Hooks</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>Hook blocking-risk flag — statically detect hook commands likely to hang (no timeout, reads stdin, long-running foreground process), since a blocking PreToolUse hook freezes the whole session.</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #6305, #10385 — hooks failing to execute/initialize with no feedback to the user</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>179</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Agents / Hooks</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>Windows-hook-syntax diagnostic — flag hook/statusLine commands using Unix-only syntax (#!/bin/sh, POSIX-only flags) that silently fail (exit 126) when spawned on native Windows.</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #62310, #93635 — statusLine/hook commands exit 126 or never execute on native Windows/Git Bash</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>180</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>UX / Interface</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>Statusline health-check button in Settings — run the configured statusLine command and show its actual output/exit code inline, cross-platform.</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #62310, #93635, #13517 — statusLine configured but never executed, no feedback</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>181</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>UX / Interface</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>Statusline editor field in Settings tab (currently unmanaged by ClAuSy) with a link noting the feature is undocumented officially.</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #5404 — statusLine feature undocumented, hard to discover</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>182</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Multi-source</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Config export/import sync bundle — bundle all detected config (settings.json, CLAUDE.md files, subagents, hooks, non-secret MCP entries) into one zip for manual multi-machine sync, since Claude Code has no built-in sync.</t>
+        </is>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>steeman.be — Syncing Claude Code Across Multiple Machines, community NAS/symlink workarounds</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>183</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Multi-source</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Cross-machine config diff tool — compare a local snapshot against a previously exported/pasted snapshot and show permission/hook/MCP differences.</t>
+        </is>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Same sync-pain research; complements the export/import bundle (#182)</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>184</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Multi-source</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Cloud-sync file-lock warning — if ~/.claude is detected inside a cloud-sync folder (OneDrive/Dropbox/Syncthing path patterns), warn about known lock conflicts on history.jsonl/.update.lock.</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>glama.ai Claude Agents MCP docs — file-lock conflicts syncing Claude config via Nextcloud/cloud sync</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>185</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D186" t="inlineStr">
+        <is>
+          <t>MCP secret-exposure scanner — extend the existing gitignored-secrets scan to check .mcp.json/.claude.json env blocks for hardcoded API keys/tokens instead of ${VAR} references.</t>
+        </is>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>Derived from MCP config-confusion cluster (#37165, #29824) — env blocks are a common place secrets leak into tracked files</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>186</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Directories</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Show whether a directory's access came from permissions.allow/additionalDirectories vs. only --add-dir (session-only, not persisted) in the Directories tab.</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #37553 — additionalDirectories vs. --add-dir behave differently for skill/dir loading</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>187</v>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Reporting</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D188" t="inlineStr">
+        <is>
+          <t>One-click copy-diagnostics button — gather a redacted bundle (Claude Code version, active settings file paths + hashes, permission mode, MCP server names only, hook command names only, all secrets stripped) formatted for pasting into a GitHub issue.</t>
+        </is>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>Complements the existing Report Confusing Config button; addresses the volume of hard-to-triage settings bugs found this round</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>188</v>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Testing / Quality</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>MCP precedence unit tests — pure-logic coverage for whatever .claude.json/.mcp.json/settings.json merge order ClAuSy implements for #163/#165, guarding against the same silent-override class of bug Claude Code itself has.</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>Self-defense against replicating GitHub #55507-style precedence bugs in ClAuSy's own merge logic</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>189</v>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>CLAUDE.md / Docs</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr">
+        <is>
+          <t>Managed-by-enterprise-policy indicator — if a managed-settings.json is present and defines a key also set in user/project settings, show which value actually wins per key (extends #176).</t>
+        </is>
+      </c>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>GitHub anthropics/claude-code #86046 — Managed.settings.json interaction confusion</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>190</v>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Newly-installed-plugin hook review prompt — when a plugin is added to a marketplace-tracked directory since ClAuSy's last scan, surface its hook definitions for one-time review before the next Claude Code session start.</t>
+        </is>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>PromptArmor marketplace-plugin hijacking disclosure — pairs with #169/#170 as an ongoing-monitoring companion</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H161"/>
   <dataValidations count="2">

</xml_diff>

<commit_message>
Mark round 5's 10 shipped feature ideas as Done in the tracking sheet
</commit_message>
<xml_diff>
--- a/ClAuSy_Feature_Ideas.xlsx
+++ b/ClAuSy_Feature_Ideas.xlsx
@@ -5606,6 +5606,16 @@
           <t>Precedence blind-spot detector: warn when defaultMode: bypassPermissions is set but a higher-precedence settings file also defines a permissions block, silently overriding it.</t>
         </is>
       </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G162" t="inlineStr">
         <is>
           <t>GitHub anthropics/claude-code #55507, #34923 — defaultMode silently dropped by permissions-block precedence merge bug</t>
@@ -5906,6 +5916,16 @@
           <t>Supply-chain hook-diff alert — when a tracked repo's .claude/settings.json hooks section changes between the last-seen commit and HEAD (e.g. after a git pull), surface a dedicated high-visibility warning distinct from the generic external-change dialog.</t>
         </is>
       </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G172" t="inlineStr">
         <is>
           <t>Check Point CVE-2025-59536 — malicious repo hooks in settings.json execute at session init before any trust prompt</t>
@@ -5966,6 +5986,16 @@
           <t>Zero-deny + bypass-mode combo alert — separate from the existing YOLO-duration banner, specifically flag the combination of bypassPermissions with an empty deny list as unusually risky.</t>
         </is>
       </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G174" t="inlineStr">
         <is>
           <t>Derived from #27040/#34923 deny-enforcement bug pattern + general bypass-mode risk reports</t>
@@ -6026,6 +6056,16 @@
           <t>Index .claude/rules/*.md files alongside CLAUDE.md in the Map tab — currently untracked, but they're a distinct doc source with the same subagent-blind-spot problem.</t>
         </is>
       </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G176" t="inlineStr">
         <is>
           <t>GitHub anthropics/claude-code #29423 — Task subagents don't load project CLAUDE.md or .claude/rules/*.md</t>
@@ -6086,6 +6126,16 @@
           <t>Subagent CLAUDE.md-blind-spot banner in Agents &amp; Routines tab — flag subagent definitions likely relying on project conventions the subagent won't see (no CLAUDE.md read instruction in description, project has a non-trivial CLAUDE.md).</t>
         </is>
       </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G178" t="inlineStr">
         <is>
           <t>GitHub anthropics/claude-code #34572, #29423 — subagents don't inherit CLAUDE.md/rules, silently apply their own interpretation</t>
@@ -6116,6 +6166,16 @@
           <t>Hook blocking-risk flag — statically detect hook commands likely to hang (no timeout, reads stdin, long-running foreground process), since a blocking PreToolUse hook freezes the whole session.</t>
         </is>
       </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G179" t="inlineStr">
         <is>
           <t>GitHub anthropics/claude-code #6305, #10385 — hooks failing to execute/initialize with no feedback to the user</t>
@@ -6146,6 +6206,16 @@
           <t>Windows-hook-syntax diagnostic — flag hook/statusLine commands using Unix-only syntax (#!/bin/sh, POSIX-only flags) that silently fail (exit 126) when spawned on native Windows.</t>
         </is>
       </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G180" t="inlineStr">
         <is>
           <t>GitHub anthropics/claude-code #62310, #93635 — statusLine/hook commands exit 126 or never execute on native Windows/Git Bash</t>
@@ -6176,6 +6246,16 @@
           <t>Statusline health-check button in Settings — run the configured statusLine command and show its actual output/exit code inline, cross-platform.</t>
         </is>
       </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G181" t="inlineStr">
         <is>
           <t>GitHub anthropics/claude-code #62310, #93635, #13517 — statusLine configured but never executed, no feedback</t>
@@ -6326,6 +6406,16 @@
           <t>MCP secret-exposure scanner — extend the existing gitignored-secrets scan to check .mcp.json/.claude.json env blocks for hardcoded API keys/tokens instead of ${VAR} references.</t>
         </is>
       </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
       <c r="G186" t="inlineStr">
         <is>
           <t>Derived from MCP config-confusion cluster (#37165, #29824) — env blocks are a common place secrets leak into tracked files</t>
@@ -6384,6 +6474,16 @@
       <c r="D188" t="inlineStr">
         <is>
           <t>One-click copy-diagnostics button — gather a redacted bundle (Claude Code version, active settings file paths + hashes, permission mode, MCP server names only, hook command names only, all secrets stripped) formatted for pasting into a GitHub issue.</t>
+        </is>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">

</xml_diff>